<commit_message>
Update transformation ramps and add conditional yamls
</commit_message>
<xml_diff>
--- a/ssp_modeling/scenario_mapping/ssp_libya_transformation_cw_20260408.xlsx
+++ b/ssp_modeling/scenario_mapping/ssp_libya_transformation_cw_20260408.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexa/Projects/ssp_libya/ssp_modeling/scenario_mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6194F4D2-0864-CC4B-B8AB-23F0D903237D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D285A6B-D103-EE4B-8D03-4AFF690DD75B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1382,7 +1382,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1403,6 +1403,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1527,7 +1533,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1741,6 +1747,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2530,14 +2539,14 @@
       </c>
       <c r="M11" s="17"/>
       <c r="N11" s="17">
-        <v>0.1</v>
+        <v>1.2</v>
       </c>
       <c r="O11" s="17">
-        <v>3</v>
+        <v>1.2</v>
       </c>
       <c r="P11" s="10">
         <f t="shared" si="1"/>
-        <v>8.0000000000000016E-2</v>
+        <v>0.96</v>
       </c>
       <c r="Q11" s="11"/>
       <c r="R11" s="11"/>
@@ -2573,14 +2582,14 @@
       </c>
       <c r="M12" s="17"/>
       <c r="N12" s="17">
-        <v>0.1</v>
+        <v>1.2</v>
       </c>
       <c r="O12" s="17">
-        <v>3</v>
+        <v>1.2</v>
       </c>
       <c r="P12" s="10">
         <f t="shared" si="1"/>
-        <v>8.0000000000000016E-2</v>
+        <v>0.96</v>
       </c>
       <c r="Q12" s="11"/>
       <c r="R12" s="11"/>
@@ -2709,11 +2718,9 @@
         <v>12</v>
       </c>
       <c r="M15" s="17"/>
-      <c r="N15" s="17">
-        <v>0.1</v>
-      </c>
+      <c r="N15" s="17"/>
       <c r="O15" s="17">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="P15" s="10" t="e">
         <f t="shared" si="1"/>
@@ -2760,7 +2767,7 @@
         <v>0.1</v>
       </c>
       <c r="O16" s="68">
-        <v>0.18</v>
+        <v>0.1</v>
       </c>
       <c r="P16" s="69">
         <f t="shared" si="1"/>
@@ -3108,7 +3115,7 @@
         <v>0.1</v>
       </c>
       <c r="O24" s="17">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="P24" s="10">
         <f t="shared" si="1"/>
@@ -3526,7 +3533,7 @@
       <c r="B35" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="C35" s="13" t="s">
+      <c r="C35" s="72" t="s">
         <v>114</v>
       </c>
       <c r="D35" s="13" t="s">
@@ -3553,7 +3560,7 @@
         <v>0.1</v>
       </c>
       <c r="O35" s="17">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="P35" s="10">
         <f t="shared" si="1"/>
@@ -3569,7 +3576,7 @@
       <c r="B36" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="C36" s="13" t="s">
+      <c r="C36" s="72" t="s">
         <v>117</v>
       </c>
       <c r="D36" s="13" t="s">
@@ -3596,7 +3603,7 @@
         <v>0.1</v>
       </c>
       <c r="O36" s="17">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="P36" s="10">
         <f t="shared" si="1"/>
@@ -3757,7 +3764,9 @@
       </c>
       <c r="M40" s="17"/>
       <c r="N40" s="17"/>
-      <c r="O40" s="17"/>
+      <c r="O40" s="17">
+        <v>1</v>
+      </c>
       <c r="P40" s="10">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3800,7 +3809,9 @@
       </c>
       <c r="M41" s="17"/>
       <c r="N41" s="17"/>
-      <c r="O41" s="17"/>
+      <c r="O41" s="17">
+        <v>1</v>
+      </c>
       <c r="P41" s="10">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3843,7 +3854,9 @@
       </c>
       <c r="M42" s="17"/>
       <c r="N42" s="17"/>
-      <c r="O42" s="17"/>
+      <c r="O42" s="17">
+        <v>1</v>
+      </c>
       <c r="P42" s="10">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3922,7 +3935,7 @@
       <c r="M44" s="17"/>
       <c r="N44" s="17"/>
       <c r="O44" s="17">
-        <v>0.05</v>
+        <v>0.8</v>
       </c>
       <c r="P44" s="10">
         <f t="shared" si="1"/>
@@ -4010,7 +4023,7 @@
       <c r="M46" s="17"/>
       <c r="N46" s="17"/>
       <c r="O46" s="17">
-        <v>0.05</v>
+        <v>0.8</v>
       </c>
       <c r="P46" s="10">
         <f t="shared" si="1"/>
@@ -4135,11 +4148,15 @@
         <v>12</v>
       </c>
       <c r="M49" s="17"/>
-      <c r="N49" s="17"/>
-      <c r="O49" s="17"/>
+      <c r="N49" s="17">
+        <v>0.3</v>
+      </c>
+      <c r="O49" s="17">
+        <v>1</v>
+      </c>
       <c r="P49" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="Q49" s="11"/>
       <c r="R49" s="11"/>

</xml_diff>

<commit_message>
update runs & tableau & cba & tornado
</commit_message>
<xml_diff>
--- a/ssp_modeling/scenario_mapping/ssp_libya_transformation_cw_20260408.xlsx
+++ b/ssp_modeling/scenario_mapping/ssp_libya_transformation_cw_20260408.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexa/Projects/ssp_libya/ssp_modeling/scenario_mapping/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabianfuentes/git/ssp_libya/ssp_modeling/scenario_mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D285A6B-D103-EE4B-8D03-4AFF690DD75B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DBA230E-C535-754A-9223-FC855622D8A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-51200" yWindow="-7160" windowWidth="25600" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -1332,8 +1332,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0%"/>
+    <numFmt numFmtId="167" formatCode="#,##0.00000"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -1533,7 +1534,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1750,6 +1751,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2411,9 +2415,9 @@
       <c r="O8" s="17">
         <v>0.1</v>
       </c>
-      <c r="P8" s="10" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+      <c r="P8" s="10">
+        <f>0.2*N8</f>
+        <v>2.0000000000000004E-2</v>
       </c>
       <c r="Q8" s="11"/>
       <c r="R8" s="11"/>
@@ -2502,7 +2506,7 @@
         <v>0.3</v>
       </c>
       <c r="P10" s="10">
-        <f t="shared" ref="P10:P63" si="1">K10*N10</f>
+        <f t="shared" ref="P10:Q63" si="1">K10*N10</f>
         <v>0.19</v>
       </c>
       <c r="Q10" s="11"/>
@@ -2539,16 +2543,19 @@
       </c>
       <c r="M11" s="17"/>
       <c r="N11" s="17">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="O11" s="17">
-        <v>1.2</v>
+        <v>1.25</v>
       </c>
       <c r="P11" s="10">
         <f t="shared" si="1"/>
-        <v>0.96</v>
-      </c>
-      <c r="Q11" s="11"/>
+        <v>0.64000000000000012</v>
+      </c>
+      <c r="Q11" s="10">
+        <f>K11*O11</f>
+        <v>1</v>
+      </c>
       <c r="R11" s="11"/>
     </row>
     <row r="12" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
@@ -2582,16 +2589,19 @@
       </c>
       <c r="M12" s="17"/>
       <c r="N12" s="17">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="O12" s="17">
-        <v>1.2</v>
+        <v>1.25</v>
       </c>
       <c r="P12" s="10">
         <f t="shared" si="1"/>
-        <v>0.96</v>
-      </c>
-      <c r="Q12" s="11"/>
+        <v>0.64000000000000012</v>
+      </c>
+      <c r="Q12" s="10">
+        <f>K12*O12</f>
+        <v>1</v>
+      </c>
       <c r="R12" s="11"/>
     </row>
     <row r="13" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
@@ -2767,7 +2777,7 @@
         <v>0.1</v>
       </c>
       <c r="O16" s="68">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="P16" s="69">
         <f t="shared" si="1"/>
@@ -3027,8 +3037,8 @@
       <c r="M22" s="17"/>
       <c r="N22" s="17"/>
       <c r="O22" s="17"/>
-      <c r="P22" s="10">
-        <f t="shared" si="1"/>
+      <c r="P22" s="73">
+        <f>K22*N22</f>
         <v>0</v>
       </c>
       <c r="Q22" s="11"/>
@@ -3112,14 +3122,14 @@
       </c>
       <c r="M24" s="17"/>
       <c r="N24" s="17">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="O24" s="17">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="P24" s="10">
         <f t="shared" si="1"/>
-        <v>2.0000000000000004E-2</v>
+        <v>0.2</v>
       </c>
       <c r="Q24" s="11"/>
       <c r="R24" s="11"/>
@@ -3238,8 +3248,12 @@
       <c r="M27" s="17">
         <v>0.1</v>
       </c>
-      <c r="N27" s="17"/>
-      <c r="O27" s="17"/>
+      <c r="N27" s="17">
+        <v>0.1</v>
+      </c>
+      <c r="O27" s="17">
+        <v>0.1</v>
+      </c>
       <c r="P27" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
@@ -3357,8 +3371,12 @@
       <c r="M30" s="17">
         <v>0.1</v>
       </c>
-      <c r="N30" s="17"/>
-      <c r="O30" s="17"/>
+      <c r="N30" s="17">
+        <v>0.1</v>
+      </c>
+      <c r="O30" s="17">
+        <v>0.1</v>
+      </c>
       <c r="P30" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
@@ -3765,7 +3783,7 @@
       <c r="M40" s="17"/>
       <c r="N40" s="17"/>
       <c r="O40" s="17">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="P40" s="10">
         <f t="shared" si="1"/>
@@ -3895,7 +3913,9 @@
       </c>
       <c r="M43" s="17"/>
       <c r="N43" s="17"/>
-      <c r="O43" s="17"/>
+      <c r="O43" s="17">
+        <v>1</v>
+      </c>
       <c r="P43" s="10">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3935,7 +3955,7 @@
       <c r="M44" s="17"/>
       <c r="N44" s="17"/>
       <c r="O44" s="17">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="P44" s="10">
         <f t="shared" si="1"/>
@@ -3979,7 +3999,9 @@
       </c>
       <c r="M45" s="17"/>
       <c r="N45" s="17"/>
-      <c r="O45" s="17"/>
+      <c r="O45" s="17">
+        <v>1</v>
+      </c>
       <c r="P45" s="10">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -4023,7 +4045,7 @@
       <c r="M46" s="17"/>
       <c r="N46" s="17"/>
       <c r="O46" s="17">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="P46" s="10">
         <f t="shared" si="1"/>
@@ -4063,7 +4085,9 @@
       </c>
       <c r="M47" s="17"/>
       <c r="N47" s="17"/>
-      <c r="O47" s="17"/>
+      <c r="O47" s="17">
+        <v>1</v>
+      </c>
       <c r="P47" s="10">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -4106,7 +4130,9 @@
       </c>
       <c r="M48" s="17"/>
       <c r="N48" s="17"/>
-      <c r="O48" s="17"/>
+      <c r="O48" s="17">
+        <v>1</v>
+      </c>
       <c r="P48" s="10">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -4149,14 +4175,14 @@
       </c>
       <c r="M49" s="17"/>
       <c r="N49" s="17">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="O49" s="17">
         <v>1</v>
       </c>
       <c r="P49" s="10">
         <f t="shared" si="1"/>
-        <v>0.09</v>
+        <v>0.15</v>
       </c>
       <c r="Q49" s="11"/>
       <c r="R49" s="11"/>
@@ -4196,7 +4222,9 @@
       </c>
       <c r="M50" s="17"/>
       <c r="N50" s="17"/>
-      <c r="O50" s="17"/>
+      <c r="O50" s="17">
+        <v>1</v>
+      </c>
       <c r="P50" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
@@ -4410,8 +4438,12 @@
       <c r="M55" s="17">
         <v>0.1</v>
       </c>
-      <c r="N55" s="17"/>
-      <c r="O55" s="17"/>
+      <c r="N55" s="17">
+        <v>0.1</v>
+      </c>
+      <c r="O55" s="17">
+        <v>0.2</v>
+      </c>
       <c r="P55" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
@@ -4493,9 +4525,7 @@
       <c r="L57" s="16">
         <v>12</v>
       </c>
-      <c r="M57" s="17">
-        <v>0.1</v>
-      </c>
+      <c r="M57" s="17"/>
       <c r="N57" s="17"/>
       <c r="O57" s="17">
         <v>1</v>

</xml_diff>

<commit_message>
gas recovery fgtv fix
</commit_message>
<xml_diff>
--- a/ssp_modeling/scenario_mapping/ssp_libya_transformation_cw_20260408.xlsx
+++ b/ssp_modeling/scenario_mapping/ssp_libya_transformation_cw_20260408.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabianfuentes/git/ssp_libya/ssp_modeling/scenario_mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{153B9434-C881-1847-9570-E5C21659B561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{802048CA-ECAE-7D48-9B5C-D1B496160CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-48540" yWindow="-7160" windowWidth="28480" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,8 +17,8 @@
     <sheet name="yaml" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">main!$A$1:$R$64</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">yaml!$A$1:$D$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">main!$A$1:$R$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">yaml!$A$1:$D$63</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="417">
   <si>
     <t>subsector</t>
   </si>
@@ -1326,6 +1326,15 @@
   </si>
   <si>
     <t>Esta impacta en waso</t>
+  </si>
+  <si>
+    <t>TX:FGTV:INC_GAS_RECOVERY</t>
+  </si>
+  <si>
+    <t>Gas Recovery</t>
+  </si>
+  <si>
+    <t>transformation_fgtv_inc_gas_recovery.yaml</t>
   </si>
 </sst>
 </file>
@@ -1335,7 +1344,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0%"/>
     <numFmt numFmtId="165" formatCode="#,##0.00000"/>
-    <numFmt numFmtId="168" formatCode="#,##0.000000"/>
+    <numFmt numFmtId="166" formatCode="#,##0.000000"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -1756,7 +1765,7 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2064,7 +2073,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:R64"/>
+  <dimension ref="A1:R65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="13.1640625" style="34" bestFit="1" customWidth="1"/>
@@ -2512,7 +2521,7 @@
         <v>0.3</v>
       </c>
       <c r="P10" s="10">
-        <f t="shared" ref="P10:P63" si="1">K10*N10</f>
+        <f t="shared" ref="P10:P64" si="1">K10*N10</f>
         <v>0.19</v>
       </c>
       <c r="Q10" s="11"/>
@@ -2526,14 +2535,12 @@
         <v>34</v>
       </c>
       <c r="C11" s="65" t="s">
-        <v>35</v>
+        <v>414</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="E11" s="13" t="s">
-        <v>242</v>
-      </c>
+        <v>415</v>
+      </c>
+      <c r="E11" s="13"/>
       <c r="F11" s="12" t="s">
         <v>243</v>
       </c>
@@ -2542,25 +2549,25 @@
       <c r="I11" s="12"/>
       <c r="J11" s="12"/>
       <c r="K11" s="19">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="L11" s="16">
         <v>12</v>
       </c>
       <c r="M11" s="17"/>
       <c r="N11" s="17">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
       <c r="O11" s="17">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="P11" s="10">
-        <f t="shared" si="1"/>
-        <v>0.64000000000000012</v>
+        <f>K11*N11</f>
+        <v>0.375</v>
       </c>
       <c r="Q11" s="10">
         <f>K11*O11</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="R11" s="11"/>
     </row>
@@ -2572,16 +2579,16 @@
         <v>34</v>
       </c>
       <c r="C12" s="65" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>244</v>
-      </c>
-      <c r="F12" s="24" t="s">
-        <v>245</v>
+        <v>242</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>243</v>
       </c>
       <c r="G12" s="12"/>
       <c r="H12" s="12"/>
@@ -2601,7 +2608,7 @@
         <v>1.25</v>
       </c>
       <c r="P12" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="P12" si="2">K12*N12</f>
         <v>0.64000000000000012</v>
       </c>
       <c r="Q12" s="10">
@@ -2615,46 +2622,43 @@
         <v>226</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" s="63" t="s">
-        <v>43</v>
-      </c>
-      <c r="E13" s="63" t="s">
-        <v>246</v>
-      </c>
-      <c r="F13" s="25" t="s">
-        <v>247</v>
+        <v>34</v>
+      </c>
+      <c r="C13" s="65" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>244</v>
+      </c>
+      <c r="F13" s="24" t="s">
+        <v>245</v>
       </c>
       <c r="G13" s="12"/>
       <c r="H13" s="12"/>
-      <c r="I13" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="J13" s="12" t="s">
-        <v>249</v>
-      </c>
-      <c r="K13" s="20">
-        <v>0.3</v>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="19">
+        <v>0.8</v>
       </c>
       <c r="L13" s="16">
         <v>12</v>
       </c>
-      <c r="M13" s="17"/>
-      <c r="N13" s="17">
-        <v>0.1</v>
-      </c>
-      <c r="O13" s="17">
+      <c r="M13" s="17">
         <v>1</v>
       </c>
+      <c r="N13" s="17"/>
+      <c r="O13" s="17"/>
       <c r="P13" s="10">
         <f t="shared" si="1"/>
-        <v>0.03</v>
-      </c>
-      <c r="Q13" s="11"/>
+        <v>0</v>
+      </c>
+      <c r="Q13" s="10">
+        <f>K13*O13</f>
+        <v>0</v>
+      </c>
       <c r="R13" s="11"/>
     </row>
     <row r="14" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
@@ -2665,27 +2669,27 @@
         <v>41</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="E14" s="13" t="s">
-        <v>250</v>
-      </c>
-      <c r="F14" s="12" t="s">
-        <v>251</v>
+        <v>42</v>
+      </c>
+      <c r="D14" s="63" t="s">
+        <v>43</v>
+      </c>
+      <c r="E14" s="63" t="s">
+        <v>246</v>
+      </c>
+      <c r="F14" s="25" t="s">
+        <v>247</v>
       </c>
       <c r="G14" s="12"/>
       <c r="H14" s="12"/>
       <c r="I14" s="12" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="J14" s="12" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="K14" s="20">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L14" s="16">
         <v>12</v>
@@ -2695,11 +2699,11 @@
         <v>0.1</v>
       </c>
       <c r="O14" s="17">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="P14" s="10">
         <f t="shared" si="1"/>
-        <v>4.0000000000000008E-2</v>
+        <v>0.03</v>
       </c>
       <c r="Q14" s="11"/>
       <c r="R14" s="11"/>
@@ -2712,128 +2716,132 @@
         <v>41</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="G15" s="12"/>
       <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="19" t="s">
-        <v>256</v>
+      <c r="I15" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="J15" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="K15" s="20">
+        <v>0.4</v>
       </c>
       <c r="L15" s="16">
         <v>12</v>
       </c>
       <c r="M15" s="17"/>
-      <c r="N15" s="17"/>
+      <c r="N15" s="17">
+        <v>0.1</v>
+      </c>
       <c r="O15" s="17">
         <v>0.5</v>
       </c>
-      <c r="P15" s="10" t="e">
+      <c r="P15" s="10">
+        <f t="shared" si="1"/>
+        <v>4.0000000000000008E-2</v>
+      </c>
+      <c r="Q15" s="11"/>
+      <c r="R15" s="11"/>
+    </row>
+    <row r="16" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>254</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="19" t="s">
+        <v>256</v>
+      </c>
+      <c r="L16" s="16">
+        <v>12</v>
+      </c>
+      <c r="M16" s="17"/>
+      <c r="N16" s="17"/>
+      <c r="O16" s="17">
+        <v>0.5</v>
+      </c>
+      <c r="P16" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-      <c r="Q15" s="11"/>
-      <c r="R15" s="11"/>
-    </row>
-    <row r="16" spans="1:18" s="71" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="65" t="s">
+      <c r="Q16" s="11"/>
+      <c r="R16" s="11"/>
+    </row>
+    <row r="17" spans="1:18" s="71" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="65" t="s">
         <v>51</v>
       </c>
-      <c r="B16" s="65" t="s">
+      <c r="B17" s="65" t="s">
         <v>51</v>
       </c>
-      <c r="C16" s="65" t="s">
+      <c r="C17" s="65" t="s">
         <v>52</v>
       </c>
-      <c r="D16" s="65" t="s">
+      <c r="D17" s="65" t="s">
         <v>53</v>
       </c>
-      <c r="E16" s="65" t="s">
+      <c r="E17" s="65" t="s">
         <v>257</v>
       </c>
-      <c r="F16" s="65" t="s">
+      <c r="F17" s="65" t="s">
         <v>258</v>
       </c>
-      <c r="G16" s="65"/>
-      <c r="H16" s="65"/>
-      <c r="I16" s="65" t="s">
+      <c r="G17" s="65"/>
+      <c r="H17" s="65"/>
+      <c r="I17" s="65" t="s">
         <v>259</v>
       </c>
-      <c r="J16" s="65" t="s">
+      <c r="J17" s="65" t="s">
         <v>260</v>
       </c>
-      <c r="K16" s="66">
+      <c r="K17" s="66">
         <v>0.5</v>
       </c>
-      <c r="L16" s="67">
-        <v>12</v>
-      </c>
-      <c r="M16" s="68"/>
-      <c r="N16" s="68">
+      <c r="L17" s="67">
+        <v>12</v>
+      </c>
+      <c r="M17" s="68"/>
+      <c r="N17" s="68">
         <v>0.1</v>
       </c>
-      <c r="O16" s="68">
+      <c r="O17" s="68">
         <v>0.5</v>
       </c>
-      <c r="P16" s="69">
+      <c r="P17" s="69">
         <f t="shared" si="1"/>
         <v>0.05</v>
       </c>
-      <c r="Q16" s="70"/>
-      <c r="R16" s="70"/>
-    </row>
-    <row r="17" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="D17" s="63" t="s">
-        <v>56</v>
-      </c>
-      <c r="E17" s="62" t="s">
-        <v>261</v>
-      </c>
-      <c r="F17" s="25" t="s">
-        <v>262</v>
-      </c>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="12" t="s">
-        <v>263</v>
-      </c>
-      <c r="J17" s="12" t="s">
-        <v>264</v>
-      </c>
-      <c r="K17" s="19">
-        <v>0.3</v>
-      </c>
-      <c r="L17" s="16">
-        <v>12</v>
-      </c>
-      <c r="M17" s="17"/>
-      <c r="N17" s="17"/>
-      <c r="O17" s="17"/>
-      <c r="P17" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q17" s="11"/>
-      <c r="R17" s="11"/>
+      <c r="Q17" s="70"/>
+      <c r="R17" s="70"/>
     </row>
     <row r="18" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="12" t="s">
@@ -2843,41 +2851,37 @@
         <v>51</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="E18" s="13" t="s">
-        <v>265</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>266</v>
+        <v>55</v>
+      </c>
+      <c r="D18" s="63" t="s">
+        <v>56</v>
+      </c>
+      <c r="E18" s="62" t="s">
+        <v>261</v>
+      </c>
+      <c r="F18" s="25" t="s">
+        <v>262</v>
       </c>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
       <c r="I18" s="12" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="J18" s="12" t="s">
-        <v>268</v>
-      </c>
-      <c r="K18" s="15">
-        <v>0.1</v>
+        <v>264</v>
+      </c>
+      <c r="K18" s="19">
+        <v>0.3</v>
       </c>
       <c r="L18" s="16">
         <v>12</v>
       </c>
       <c r="M18" s="17"/>
-      <c r="N18" s="17">
-        <v>0.1</v>
-      </c>
-      <c r="O18" s="17">
-        <v>1</v>
-      </c>
+      <c r="N18" s="17"/>
+      <c r="O18" s="17"/>
       <c r="P18" s="10">
         <f t="shared" si="1"/>
-        <v>1.0000000000000002E-2</v>
+        <v>0</v>
       </c>
       <c r="Q18" s="11"/>
       <c r="R18" s="11"/>
@@ -2890,21 +2894,25 @@
         <v>51</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="G19" s="12"/>
       <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
+      <c r="I19" s="12" t="s">
+        <v>267</v>
+      </c>
+      <c r="J19" s="12" t="s">
+        <v>268</v>
+      </c>
       <c r="K19" s="15">
         <v>0.1</v>
       </c>
@@ -2912,11 +2920,15 @@
         <v>12</v>
       </c>
       <c r="M19" s="17"/>
-      <c r="N19" s="17"/>
-      <c r="O19" s="17"/>
+      <c r="N19" s="17">
+        <v>0.1</v>
+      </c>
+      <c r="O19" s="17">
+        <v>1</v>
+      </c>
       <c r="P19" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.0000000000000002E-2</v>
       </c>
       <c r="Q19" s="11"/>
       <c r="R19" s="11"/>
@@ -2929,16 +2941,16 @@
         <v>51</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="G20" s="12"/>
       <c r="H20" s="12"/>
@@ -2951,15 +2963,11 @@
         <v>12</v>
       </c>
       <c r="M20" s="17"/>
-      <c r="N20" s="17">
-        <v>0.1</v>
-      </c>
-      <c r="O20" s="17">
-        <v>0.5</v>
-      </c>
+      <c r="N20" s="17"/>
+      <c r="O20" s="17"/>
       <c r="P20" s="10">
         <f t="shared" si="1"/>
-        <v>1.0000000000000002E-2</v>
+        <v>0</v>
       </c>
       <c r="Q20" s="11"/>
       <c r="R20" s="11"/>
@@ -2972,16 +2980,16 @@
         <v>51</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="G21" s="12"/>
       <c r="H21" s="12"/>
@@ -3009,52 +3017,45 @@
     </row>
     <row r="22" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">
-        <v>212</v>
+        <v>51</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="D22" s="63" t="s">
-        <v>72</v>
-      </c>
-      <c r="E22" s="62" t="s">
-        <v>275</v>
-      </c>
-      <c r="F22" s="25" t="s">
-        <v>276</v>
+        <v>67</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>273</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>274</v>
       </c>
       <c r="G22" s="12"/>
       <c r="H22" s="12"/>
-      <c r="I22" s="13" t="s">
-        <v>277</v>
-      </c>
-      <c r="J22" s="13" t="s">
-        <v>278</v>
-      </c>
+      <c r="I22" s="12"/>
+      <c r="J22" s="12"/>
       <c r="K22" s="15">
-        <v>0.999</v>
+        <v>0.1</v>
       </c>
       <c r="L22" s="16">
         <v>12</v>
       </c>
       <c r="M22" s="17"/>
       <c r="N22" s="17">
-        <v>0.89</v>
+        <v>0.1</v>
       </c>
       <c r="O22" s="17">
-        <v>0.98999899999999996</v>
-      </c>
-      <c r="P22" s="73">
-        <f>K22*N22</f>
-        <v>0.88911000000000007</v>
-      </c>
-      <c r="Q22" s="74">
-        <f>K22*O22</f>
-        <v>0.989009001</v>
-      </c>
+        <v>0.5</v>
+      </c>
+      <c r="P22" s="10">
+        <f t="shared" si="1"/>
+        <v>1.0000000000000002E-2</v>
+      </c>
+      <c r="Q22" s="11"/>
       <c r="R22" s="11"/>
     </row>
     <row r="23" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
@@ -3065,39 +3066,46 @@
         <v>70</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="D23" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="E23" s="13" t="s">
-        <v>279</v>
-      </c>
-      <c r="F23" s="12" t="s">
-        <v>280</v>
+        <v>71</v>
+      </c>
+      <c r="D23" s="63" t="s">
+        <v>72</v>
+      </c>
+      <c r="E23" s="62" t="s">
+        <v>275</v>
+      </c>
+      <c r="F23" s="25" t="s">
+        <v>276</v>
       </c>
       <c r="G23" s="12"/>
       <c r="H23" s="12"/>
-      <c r="I23" s="12" t="s">
-        <v>281</v>
-      </c>
-      <c r="J23" s="26" t="s">
-        <v>282</v>
-      </c>
-      <c r="K23" s="19">
-        <v>0.95</v>
+      <c r="I23" s="13" t="s">
+        <v>277</v>
+      </c>
+      <c r="J23" s="13" t="s">
+        <v>278</v>
+      </c>
+      <c r="K23" s="15">
+        <v>0.999</v>
       </c>
       <c r="L23" s="16">
         <v>12</v>
       </c>
       <c r="M23" s="17"/>
-      <c r="N23" s="17"/>
-      <c r="O23" s="17"/>
-      <c r="P23" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q23" s="11"/>
+      <c r="N23" s="17">
+        <v>0.89</v>
+      </c>
+      <c r="O23" s="17">
+        <v>0.98999899999999996</v>
+      </c>
+      <c r="P23" s="73">
+        <f>K23*N23</f>
+        <v>0.88911000000000007</v>
+      </c>
+      <c r="Q23" s="74">
+        <f>K23*O23</f>
+        <v>0.989009001</v>
+      </c>
       <c r="R23" s="11"/>
     </row>
     <row r="24" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
@@ -3108,46 +3116,39 @@
         <v>70</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="D24" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="E24" s="62" t="s">
-        <v>283</v>
-      </c>
-      <c r="F24" s="25" t="s">
-        <v>284</v>
+        <v>74</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>279</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>280</v>
       </c>
       <c r="G24" s="12"/>
       <c r="H24" s="12"/>
-      <c r="I24" s="13" t="s">
-        <v>285</v>
-      </c>
-      <c r="J24" s="13" t="s">
-        <v>286</v>
-      </c>
-      <c r="K24" s="15">
-        <v>0.2</v>
+      <c r="I24" s="12" t="s">
+        <v>281</v>
+      </c>
+      <c r="J24" s="26" t="s">
+        <v>282</v>
+      </c>
+      <c r="K24" s="19">
+        <v>0.95</v>
       </c>
       <c r="L24" s="16">
         <v>12</v>
       </c>
       <c r="M24" s="17"/>
-      <c r="N24" s="17">
-        <v>1</v>
-      </c>
-      <c r="O24" s="17">
-        <v>4.9899899999999997</v>
-      </c>
+      <c r="N24" s="17"/>
+      <c r="O24" s="17"/>
       <c r="P24" s="10">
-        <f>K24*N24</f>
-        <v>0.2</v>
-      </c>
-      <c r="Q24" s="74">
-        <f>K24*O24</f>
-        <v>0.99799799999999994</v>
-      </c>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q24" s="11"/>
       <c r="R24" s="11"/>
     </row>
     <row r="25" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
@@ -3158,66 +3159,77 @@
         <v>70</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="D25" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="E25" s="13" t="s">
-        <v>287</v>
-      </c>
-      <c r="F25" s="12" t="s">
-        <v>288</v>
+        <v>77</v>
+      </c>
+      <c r="D25" s="63" t="s">
+        <v>78</v>
+      </c>
+      <c r="E25" s="62" t="s">
+        <v>283</v>
+      </c>
+      <c r="F25" s="25" t="s">
+        <v>284</v>
       </c>
       <c r="G25" s="12"/>
       <c r="H25" s="12"/>
-      <c r="I25" s="12" t="s">
-        <v>289</v>
-      </c>
-      <c r="J25" s="12" t="s">
-        <v>290</v>
-      </c>
-      <c r="K25" s="19">
-        <v>0.1</v>
+      <c r="I25" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="J25" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="K25" s="15">
+        <v>0.2</v>
       </c>
       <c r="L25" s="16">
         <v>12</v>
       </c>
       <c r="M25" s="17"/>
-      <c r="N25" s="17"/>
-      <c r="O25" s="17"/>
+      <c r="N25" s="17">
+        <v>1</v>
+      </c>
+      <c r="O25" s="17">
+        <v>4.9899899999999997</v>
+      </c>
       <c r="P25" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q25" s="11"/>
+        <f>K25*N25</f>
+        <v>0.2</v>
+      </c>
+      <c r="Q25" s="74">
+        <f>K25*O25</f>
+        <v>0.99799799999999994</v>
+      </c>
       <c r="R25" s="11"/>
     </row>
-    <row r="26" spans="1:18" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="12" t="s">
         <v>212</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G26" s="12"/>
       <c r="H26" s="12"/>
-      <c r="I26" s="12"/>
-      <c r="J26" s="12"/>
+      <c r="I26" s="12" t="s">
+        <v>289</v>
+      </c>
+      <c r="J26" s="12" t="s">
+        <v>290</v>
+      </c>
       <c r="K26" s="19">
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
       <c r="L26" s="16">
         <v>12</v>
@@ -3230,9 +3242,9 @@
         <v>0</v>
       </c>
       <c r="Q26" s="11"/>
-      <c r="R26" s="28"/>
-    </row>
-    <row r="27" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R26" s="11"/>
+    </row>
+    <row r="27" spans="1:18" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="12" t="s">
         <v>212</v>
       </c>
@@ -3240,40 +3252,36 @@
         <v>83</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="G27" s="12"/>
       <c r="H27" s="12"/>
       <c r="I27" s="12"/>
       <c r="J27" s="12"/>
-      <c r="K27" s="19" t="s">
-        <v>295</v>
+      <c r="K27" s="19">
+        <v>0.9</v>
       </c>
       <c r="L27" s="16">
         <v>12</v>
       </c>
       <c r="M27" s="17"/>
-      <c r="N27" s="17">
-        <v>0.1</v>
-      </c>
-      <c r="O27" s="17">
-        <v>0.1</v>
-      </c>
-      <c r="P27" s="10" t="e">
+      <c r="N27" s="17"/>
+      <c r="O27" s="17"/>
+      <c r="P27" s="10">
         <f t="shared" si="1"/>
-        <v>#VALUE!</v>
+        <v>0</v>
       </c>
       <c r="Q27" s="11"/>
-      <c r="R27" s="11"/>
+      <c r="R27" s="28"/>
     </row>
     <row r="28" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="12" t="s">
@@ -3283,13 +3291,13 @@
         <v>83</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="F28" s="12" t="s">
         <v>294</v>
@@ -3299,14 +3307,18 @@
       <c r="I28" s="12"/>
       <c r="J28" s="12"/>
       <c r="K28" s="19" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="L28" s="16">
         <v>12</v>
       </c>
       <c r="M28" s="17"/>
-      <c r="N28" s="17"/>
-      <c r="O28" s="17"/>
+      <c r="N28" s="17">
+        <v>0.1</v>
+      </c>
+      <c r="O28" s="17">
+        <v>0.1</v>
+      </c>
       <c r="P28" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
@@ -3322,13 +3334,13 @@
         <v>83</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="F29" s="12" t="s">
         <v>294</v>
@@ -3338,7 +3350,7 @@
       <c r="I29" s="12"/>
       <c r="J29" s="12"/>
       <c r="K29" s="19" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="L29" s="16">
         <v>12</v>
@@ -3358,37 +3370,33 @@
         <v>212</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
       <c r="J30" s="12"/>
-      <c r="K30" s="15" t="s">
-        <v>302</v>
+      <c r="K30" s="19" t="s">
+        <v>299</v>
       </c>
       <c r="L30" s="16">
         <v>12</v>
       </c>
       <c r="M30" s="17"/>
-      <c r="N30" s="17">
-        <v>0.1</v>
-      </c>
-      <c r="O30" s="17">
-        <v>0.1</v>
-      </c>
+      <c r="N30" s="17"/>
+      <c r="O30" s="17"/>
       <c r="P30" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
@@ -3404,38 +3412,42 @@
         <v>96</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="F31" s="12" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="G31" s="12"/>
       <c r="H31" s="12"/>
       <c r="I31" s="12"/>
       <c r="J31" s="12"/>
-      <c r="K31" s="19">
-        <v>0.5</v>
+      <c r="K31" s="15" t="s">
+        <v>302</v>
       </c>
       <c r="L31" s="16">
         <v>12</v>
       </c>
       <c r="M31" s="17"/>
-      <c r="N31" s="17"/>
-      <c r="O31" s="17"/>
-      <c r="P31" s="10">
+      <c r="N31" s="17">
+        <v>0.1</v>
+      </c>
+      <c r="O31" s="17">
+        <v>0.1</v>
+      </c>
+      <c r="P31" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="Q31" s="11"/>
       <c r="R31" s="11"/>
     </row>
-    <row r="32" spans="1:18" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="12" t="s">
         <v>212</v>
       </c>
@@ -3443,27 +3455,23 @@
         <v>96</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="G32" s="12"/>
       <c r="H32" s="12"/>
-      <c r="I32" s="12" t="s">
-        <v>307</v>
-      </c>
-      <c r="J32" s="12" t="s">
-        <v>308</v>
-      </c>
+      <c r="I32" s="12"/>
+      <c r="J32" s="12"/>
       <c r="K32" s="19">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="L32" s="16">
         <v>12</v>
@@ -3475,34 +3483,38 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Q32" s="17"/>
-      <c r="R32" s="29"/>
-    </row>
-    <row r="33" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q32" s="11"/>
+      <c r="R32" s="11"/>
+    </row>
+    <row r="33" spans="1:18" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="12" t="s">
-        <v>309</v>
+        <v>212</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="F33" s="12" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="G33" s="12"/>
       <c r="H33" s="12"/>
-      <c r="I33" s="12"/>
-      <c r="J33" s="12"/>
+      <c r="I33" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="J33" s="12" t="s">
+        <v>308</v>
+      </c>
       <c r="K33" s="19">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="L33" s="16">
         <v>12</v>
@@ -3514,8 +3526,8 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Q33" s="11"/>
-      <c r="R33" s="11"/>
+      <c r="Q33" s="17"/>
+      <c r="R33" s="29"/>
     </row>
     <row r="34" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="12" t="s">
@@ -3525,23 +3537,23 @@
         <v>106</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="G34" s="12"/>
       <c r="H34" s="12"/>
       <c r="I34" s="12"/>
       <c r="J34" s="12"/>
       <c r="K34" s="19">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="L34" s="16">
         <v>12</v>
@@ -3558,43 +3570,39 @@
     </row>
     <row r="35" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="12" t="s">
-        <v>226</v>
+        <v>309</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="C35" s="72" t="s">
-        <v>114</v>
+        <v>106</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>110</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="F35" s="12" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="G35" s="12"/>
       <c r="H35" s="12"/>
       <c r="I35" s="12"/>
       <c r="J35" s="12"/>
-      <c r="K35" s="20">
-        <v>0.5</v>
+      <c r="K35" s="19">
+        <v>0.9</v>
       </c>
       <c r="L35" s="16">
         <v>12</v>
       </c>
       <c r="M35" s="17"/>
-      <c r="N35" s="17">
-        <v>0.1</v>
-      </c>
-      <c r="O35" s="17">
-        <v>0.5</v>
-      </c>
+      <c r="N35" s="17"/>
+      <c r="O35" s="17"/>
       <c r="P35" s="10">
         <f t="shared" si="1"/>
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="Q35" s="11"/>
       <c r="R35" s="11"/>
@@ -3607,22 +3615,22 @@
         <v>113</v>
       </c>
       <c r="C36" s="72" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="F36" s="12" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="G36" s="12"/>
       <c r="H36" s="12"/>
       <c r="I36" s="12"/>
       <c r="J36" s="12"/>
-      <c r="K36" s="19">
+      <c r="K36" s="20">
         <v>0.5</v>
       </c>
       <c r="L36" s="16">
@@ -3649,63 +3657,67 @@
       <c r="B37" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="C37" s="13" t="s">
-        <v>120</v>
+      <c r="C37" s="72" t="s">
+        <v>117</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="F37" s="12" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="G37" s="12"/>
       <c r="H37" s="12"/>
       <c r="I37" s="12"/>
       <c r="J37" s="12"/>
-      <c r="K37" s="20">
-        <v>0.95</v>
+      <c r="K37" s="19">
+        <v>0.5</v>
       </c>
       <c r="L37" s="16">
         <v>12</v>
       </c>
       <c r="M37" s="17"/>
-      <c r="N37" s="17"/>
-      <c r="O37" s="17"/>
+      <c r="N37" s="17">
+        <v>0.1</v>
+      </c>
+      <c r="O37" s="17">
+        <v>0.5</v>
+      </c>
       <c r="P37" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="Q37" s="11"/>
       <c r="R37" s="11"/>
     </row>
     <row r="38" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="12" t="s">
-        <v>212</v>
+        <v>226</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="F38" s="12" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="G38" s="12"/>
       <c r="H38" s="12"/>
       <c r="I38" s="12"/>
       <c r="J38" s="12"/>
-      <c r="K38" s="19">
-        <v>0.2</v>
+      <c r="K38" s="20">
+        <v>0.95</v>
       </c>
       <c r="L38" s="16">
         <v>12</v>
@@ -3728,16 +3740,16 @@
         <v>123</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E39" s="13" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="F39" s="12" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="G39" s="12"/>
       <c r="H39" s="12"/>
@@ -3761,42 +3773,36 @@
     </row>
     <row r="40" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="12" t="s">
-        <v>226</v>
+        <v>212</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="F40" s="12" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="G40" s="12"/>
       <c r="H40" s="12"/>
-      <c r="I40" s="12" t="s">
-        <v>326</v>
-      </c>
-      <c r="J40" s="12" t="s">
-        <v>327</v>
-      </c>
+      <c r="I40" s="12"/>
+      <c r="J40" s="12"/>
       <c r="K40" s="19">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="L40" s="16">
         <v>12</v>
       </c>
       <c r="M40" s="17"/>
       <c r="N40" s="17"/>
-      <c r="O40" s="17">
-        <v>1.5</v>
-      </c>
+      <c r="O40" s="17"/>
       <c r="P40" s="10">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -3809,27 +3815,27 @@
         <v>226</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="F41" s="12" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="G41" s="12"/>
-      <c r="H41" s="30"/>
+      <c r="H41" s="12"/>
       <c r="I41" s="12" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="J41" s="12" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="K41" s="19">
         <v>0.25</v>
@@ -3840,7 +3846,7 @@
       <c r="M41" s="17"/>
       <c r="N41" s="17"/>
       <c r="O41" s="17">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="P41" s="10">
         <f t="shared" si="1"/>
@@ -3849,7 +3855,7 @@
       <c r="Q41" s="11"/>
       <c r="R41" s="11"/>
     </row>
-    <row r="42" spans="1:18" s="4" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="12" t="s">
         <v>226</v>
       </c>
@@ -3857,24 +3863,24 @@
         <v>134</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="F42" s="12" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="G42" s="12"/>
       <c r="H42" s="30"/>
       <c r="I42" s="12" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="J42" s="12" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="K42" s="19">
         <v>0.25</v>
@@ -3888,13 +3894,13 @@
         <v>1</v>
       </c>
       <c r="P42" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>K42*O42</f>
+        <v>0.25</v>
       </c>
       <c r="Q42" s="11"/>
       <c r="R42" s="11"/>
     </row>
-    <row r="43" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:18" s="4" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="12" t="s">
         <v>226</v>
       </c>
@@ -3902,21 +3908,25 @@
         <v>134</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="F43" s="12" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="G43" s="12"/>
-      <c r="H43" s="12"/>
-      <c r="I43" s="12"/>
-      <c r="J43" s="12"/>
+      <c r="H43" s="30"/>
+      <c r="I43" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="J43" s="12" t="s">
+        <v>335</v>
+      </c>
       <c r="K43" s="19">
         <v>0.25</v>
       </c>
@@ -3929,8 +3939,8 @@
         <v>1</v>
       </c>
       <c r="P43" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" ref="P43:P50" si="3">K43*O43</f>
+        <v>0.25</v>
       </c>
       <c r="Q43" s="11"/>
       <c r="R43" s="11"/>
@@ -3943,23 +3953,23 @@
         <v>134</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="F44" s="12" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="G44" s="12"/>
       <c r="H44" s="12"/>
       <c r="I44" s="12"/>
       <c r="J44" s="12"/>
       <c r="K44" s="19">
-        <v>0.7</v>
+        <v>0.25</v>
       </c>
       <c r="L44" s="16">
         <v>12</v>
@@ -3970,8 +3980,8 @@
         <v>1</v>
       </c>
       <c r="P44" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>0.25</v>
       </c>
       <c r="Q44" s="11"/>
       <c r="R44" s="11"/>
@@ -3984,25 +3994,21 @@
         <v>134</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="F45" s="12" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="G45" s="12"/>
       <c r="H45" s="12"/>
-      <c r="I45" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="J45" s="12" t="s">
-        <v>343</v>
-      </c>
+      <c r="I45" s="12"/>
+      <c r="J45" s="12"/>
       <c r="K45" s="19">
         <v>0.7</v>
       </c>
@@ -4015,8 +4021,8 @@
         <v>1</v>
       </c>
       <c r="P45" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>0.7</v>
       </c>
       <c r="Q45" s="11"/>
       <c r="R45" s="11"/>
@@ -4029,26 +4035,26 @@
         <v>134</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="F46" s="12" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="G46" s="12"/>
       <c r="H46" s="12"/>
       <c r="I46" s="12" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="J46" s="12" t="s">
-        <v>347</v>
-      </c>
-      <c r="K46" s="20">
+        <v>343</v>
+      </c>
+      <c r="K46" s="19">
         <v>0.7</v>
       </c>
       <c r="L46" s="16">
@@ -4060,8 +4066,8 @@
         <v>1</v>
       </c>
       <c r="P46" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>0.7</v>
       </c>
       <c r="Q46" s="11"/>
       <c r="R46" s="11"/>
@@ -4074,23 +4080,27 @@
         <v>134</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="F47" s="12" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="G47" s="12"/>
       <c r="H47" s="12"/>
-      <c r="I47" s="12"/>
-      <c r="J47" s="12"/>
-      <c r="K47" s="19">
-        <v>0.25</v>
+      <c r="I47" s="12" t="s">
+        <v>346</v>
+      </c>
+      <c r="J47" s="12" t="s">
+        <v>347</v>
+      </c>
+      <c r="K47" s="20">
+        <v>0.7</v>
       </c>
       <c r="L47" s="16">
         <v>12</v>
@@ -4101,8 +4111,8 @@
         <v>1</v>
       </c>
       <c r="P47" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>0.7</v>
       </c>
       <c r="Q47" s="11"/>
       <c r="R47" s="11"/>
@@ -4115,38 +4125,32 @@
         <v>134</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="F48" s="12" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="G48" s="12"/>
       <c r="H48" s="12"/>
-      <c r="I48" s="12" t="s">
-        <v>352</v>
-      </c>
-      <c r="J48" s="12" t="s">
-        <v>353</v>
-      </c>
+      <c r="I48" s="12"/>
+      <c r="J48" s="12"/>
       <c r="K48" s="19">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="L48" s="16">
         <v>12</v>
       </c>
       <c r="M48" s="17"/>
       <c r="N48" s="17"/>
-      <c r="O48" s="17">
-        <v>1</v>
-      </c>
+      <c r="O48" s="17"/>
       <c r="P48" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="Q48" s="11"/>
@@ -4160,41 +4164,39 @@
         <v>134</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="F49" s="12" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="G49" s="12"/>
       <c r="H49" s="12"/>
       <c r="I49" s="12" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="J49" s="12" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="K49" s="19">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L49" s="16">
         <v>12</v>
       </c>
       <c r="M49" s="17"/>
-      <c r="N49" s="17">
-        <v>0.5</v>
-      </c>
+      <c r="N49" s="17"/>
       <c r="O49" s="17">
         <v>1</v>
       </c>
       <c r="P49" s="10">
-        <f t="shared" si="1"/>
-        <v>0.15</v>
+        <f t="shared" si="3"/>
+        <v>0.2</v>
       </c>
       <c r="Q49" s="11"/>
       <c r="R49" s="11"/>
@@ -4207,79 +4209,84 @@
         <v>134</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="F50" s="12" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="G50" s="12"/>
       <c r="H50" s="12"/>
       <c r="I50" s="12" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="J50" s="12" t="s">
-        <v>361</v>
-      </c>
-      <c r="K50" s="19" t="s">
-        <v>362</v>
+        <v>357</v>
+      </c>
+      <c r="K50" s="19">
+        <v>0.3</v>
       </c>
       <c r="L50" s="16">
         <v>12</v>
       </c>
       <c r="M50" s="17"/>
-      <c r="N50" s="17"/>
+      <c r="N50" s="17">
+        <v>0.5</v>
+      </c>
       <c r="O50" s="17">
         <v>1</v>
       </c>
-      <c r="P50" s="10" t="e">
-        <f t="shared" si="1"/>
-        <v>#VALUE!</v>
+      <c r="P50" s="10">
+        <f t="shared" si="3"/>
+        <v>0.3</v>
       </c>
       <c r="Q50" s="11"/>
       <c r="R50" s="11"/>
     </row>
     <row r="51" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="12" t="s">
-        <v>51</v>
+        <v>226</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>165</v>
+        <v>134</v>
       </c>
       <c r="C51" s="13" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D51" s="13" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="F51" s="12" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="G51" s="12"/>
       <c r="H51" s="12"/>
-      <c r="I51" s="12"/>
-      <c r="J51" s="12"/>
-      <c r="K51" s="19">
-        <v>0.85</v>
+      <c r="I51" s="12" t="s">
+        <v>360</v>
+      </c>
+      <c r="J51" s="12" t="s">
+        <v>361</v>
+      </c>
+      <c r="K51" s="19" t="s">
+        <v>362</v>
       </c>
       <c r="L51" s="16">
         <v>12</v>
       </c>
       <c r="M51" s="17"/>
       <c r="N51" s="17"/>
-      <c r="O51" s="17"/>
-      <c r="P51" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="O51" s="17">
+        <v>1</v>
+      </c>
+      <c r="P51" s="10"/>
       <c r="Q51" s="11"/>
       <c r="R51" s="11"/>
     </row>
@@ -4291,36 +4298,30 @@
         <v>165</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="E52" s="13" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="F52" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="G52" s="12"/>
       <c r="H52" s="12"/>
-      <c r="I52" s="12" t="s">
-        <v>367</v>
-      </c>
-      <c r="J52" s="12" t="s">
-        <v>368</v>
-      </c>
+      <c r="I52" s="12"/>
+      <c r="J52" s="12"/>
       <c r="K52" s="19">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="L52" s="16">
         <v>12</v>
       </c>
       <c r="M52" s="17"/>
       <c r="N52" s="17"/>
-      <c r="O52" s="17">
-        <v>0.5</v>
-      </c>
+      <c r="O52" s="17"/>
       <c r="P52" s="10">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -4330,43 +4331,45 @@
     </row>
     <row r="53" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="12" t="s">
-        <v>369</v>
+        <v>51</v>
       </c>
       <c r="B53" s="13" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="C53" s="13" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="D53" s="13" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="E53" s="13" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="F53" s="12" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="G53" s="12"/>
       <c r="H53" s="12"/>
       <c r="I53" s="12" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="J53" s="12" t="s">
-        <v>373</v>
-      </c>
-      <c r="K53" s="19" t="s">
-        <v>374</v>
+        <v>368</v>
+      </c>
+      <c r="K53" s="19">
+        <v>0.9</v>
       </c>
       <c r="L53" s="16">
         <v>12</v>
       </c>
       <c r="M53" s="17"/>
       <c r="N53" s="17"/>
-      <c r="O53" s="17"/>
-      <c r="P53" s="10" t="e">
+      <c r="O53" s="17">
+        <v>0.5</v>
+      </c>
+      <c r="P53" s="10">
         <f t="shared" si="1"/>
-        <v>#VALUE!</v>
+        <v>0</v>
       </c>
       <c r="Q53" s="11"/>
       <c r="R53" s="11"/>
@@ -4379,13 +4382,13 @@
         <v>172</v>
       </c>
       <c r="C54" s="13" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D54" s="13" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="E54" s="13" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="F54" s="12" t="s">
         <v>371</v>
@@ -4393,13 +4396,13 @@
       <c r="G54" s="12"/>
       <c r="H54" s="12"/>
       <c r="I54" s="12" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="J54" s="12" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="K54" s="19" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="L54" s="16">
         <v>12</v>
@@ -4422,13 +4425,13 @@
         <v>172</v>
       </c>
       <c r="C55" s="13" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="D55" s="13" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="E55" s="13" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="F55" s="12" t="s">
         <v>371</v>
@@ -4436,24 +4439,20 @@
       <c r="G55" s="12"/>
       <c r="H55" s="12"/>
       <c r="I55" s="12" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="J55" s="12" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="K55" s="19" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="L55" s="16">
         <v>12</v>
       </c>
       <c r="M55" s="17"/>
-      <c r="N55" s="17">
-        <v>0.1</v>
-      </c>
-      <c r="O55" s="17">
-        <v>0.2</v>
-      </c>
+      <c r="N55" s="17"/>
+      <c r="O55" s="17"/>
       <c r="P55" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
@@ -4466,42 +4465,44 @@
         <v>369</v>
       </c>
       <c r="B56" s="13" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D56" s="13" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="E56" s="13" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="F56" s="12" t="s">
-        <v>384</v>
+        <v>371</v>
       </c>
       <c r="G56" s="12"/>
       <c r="H56" s="12"/>
       <c r="I56" s="12" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="J56" s="12" t="s">
-        <v>386</v>
-      </c>
-      <c r="K56" s="19">
-        <v>0.3</v>
+        <v>381</v>
+      </c>
+      <c r="K56" s="19" t="s">
+        <v>382</v>
       </c>
       <c r="L56" s="16">
         <v>12</v>
       </c>
       <c r="M56" s="17"/>
-      <c r="N56" s="17"/>
+      <c r="N56" s="17">
+        <v>0.1</v>
+      </c>
       <c r="O56" s="17">
-        <v>1</v>
-      </c>
-      <c r="P56" s="10">
+        <v>0.2</v>
+      </c>
+      <c r="P56" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="Q56" s="11"/>
       <c r="R56" s="11"/>
@@ -4514,23 +4515,27 @@
         <v>182</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D57" s="13" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="E57" s="13" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="F57" s="12" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="G57" s="12"/>
       <c r="H57" s="12"/>
-      <c r="I57" s="12"/>
-      <c r="J57" s="12"/>
-      <c r="K57" s="15" t="s">
-        <v>389</v>
+      <c r="I57" s="12" t="s">
+        <v>385</v>
+      </c>
+      <c r="J57" s="12" t="s">
+        <v>386</v>
+      </c>
+      <c r="K57" s="19">
+        <v>0.3</v>
       </c>
       <c r="L57" s="16">
         <v>12</v>
@@ -4540,9 +4545,9 @@
       <c r="O57" s="17">
         <v>1</v>
       </c>
-      <c r="P57" s="10" t="e">
+      <c r="P57" s="10">
         <f t="shared" si="1"/>
-        <v>#VALUE!</v>
+        <v>0</v>
       </c>
       <c r="Q57" s="11"/>
       <c r="R57" s="11"/>
@@ -4555,27 +4560,23 @@
         <v>182</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>189</v>
-      </c>
-      <c r="D58" s="62" t="s">
-        <v>167</v>
-      </c>
-      <c r="E58" s="62" t="s">
-        <v>390</v>
-      </c>
-      <c r="F58" s="22" t="s">
-        <v>391</v>
+        <v>186</v>
+      </c>
+      <c r="D58" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="E58" s="13" t="s">
+        <v>387</v>
+      </c>
+      <c r="F58" s="12" t="s">
+        <v>388</v>
       </c>
       <c r="G58" s="12"/>
       <c r="H58" s="12"/>
-      <c r="I58" s="12" t="s">
-        <v>392</v>
-      </c>
-      <c r="J58" s="12" t="s">
-        <v>393</v>
-      </c>
-      <c r="K58" s="15">
-        <v>0.85</v>
+      <c r="I58" s="12"/>
+      <c r="J58" s="12"/>
+      <c r="K58" s="15" t="s">
+        <v>389</v>
       </c>
       <c r="L58" s="16">
         <v>12</v>
@@ -4583,11 +4584,11 @@
       <c r="M58" s="17"/>
       <c r="N58" s="17"/>
       <c r="O58" s="17">
-        <v>0.1</v>
-      </c>
-      <c r="P58" s="10">
+        <v>1</v>
+      </c>
+      <c r="P58" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="Q58" s="11"/>
       <c r="R58" s="11"/>
@@ -4600,21 +4601,25 @@
         <v>182</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="D59" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="E59" s="13" t="s">
-        <v>394</v>
-      </c>
-      <c r="F59" s="12" t="s">
-        <v>395</v>
+        <v>189</v>
+      </c>
+      <c r="D59" s="62" t="s">
+        <v>167</v>
+      </c>
+      <c r="E59" s="62" t="s">
+        <v>390</v>
+      </c>
+      <c r="F59" s="22" t="s">
+        <v>391</v>
       </c>
       <c r="G59" s="12"/>
       <c r="H59" s="12"/>
-      <c r="I59" s="12"/>
-      <c r="J59" s="12"/>
+      <c r="I59" s="12" t="s">
+        <v>392</v>
+      </c>
+      <c r="J59" s="12" t="s">
+        <v>393</v>
+      </c>
       <c r="K59" s="15">
         <v>0.85</v>
       </c>
@@ -4624,7 +4629,7 @@
       <c r="M59" s="17"/>
       <c r="N59" s="17"/>
       <c r="O59" s="17">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="P59" s="10">
         <f t="shared" si="1"/>
@@ -4641,16 +4646,16 @@
         <v>182</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D60" s="13" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="E60" s="13" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="F60" s="12" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="G60" s="12"/>
       <c r="H60" s="12"/>
@@ -4664,7 +4669,9 @@
       </c>
       <c r="M60" s="17"/>
       <c r="N60" s="17"/>
-      <c r="O60" s="17"/>
+      <c r="O60" s="17">
+        <v>0.15</v>
+      </c>
       <c r="P60" s="10">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -4673,43 +4680,37 @@
       <c r="R60" s="11"/>
     </row>
     <row r="61" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="40" t="s">
+      <c r="A61" s="12" t="s">
         <v>369</v>
       </c>
-      <c r="B61" s="64" t="s">
+      <c r="B61" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="C61" s="64" t="s">
-        <v>197</v>
-      </c>
-      <c r="D61" s="64" t="s">
-        <v>198</v>
-      </c>
-      <c r="E61" s="64" t="s">
-        <v>398</v>
-      </c>
-      <c r="F61" s="40" t="s">
-        <v>399</v>
-      </c>
-      <c r="G61" s="40"/>
-      <c r="H61" s="40"/>
-      <c r="I61" s="40" t="s">
-        <v>400</v>
-      </c>
-      <c r="J61" s="40" t="s">
-        <v>401</v>
-      </c>
-      <c r="K61" s="41">
-        <v>1</v>
-      </c>
-      <c r="L61" s="42">
-        <v>12</v>
-      </c>
-      <c r="M61" s="43"/>
-      <c r="N61" s="43"/>
-      <c r="O61" s="43">
-        <v>1</v>
-      </c>
+      <c r="C61" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="D61" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="E61" s="13" t="s">
+        <v>396</v>
+      </c>
+      <c r="F61" s="12" t="s">
+        <v>397</v>
+      </c>
+      <c r="G61" s="12"/>
+      <c r="H61" s="12"/>
+      <c r="I61" s="12"/>
+      <c r="J61" s="12"/>
+      <c r="K61" s="15">
+        <v>0.85</v>
+      </c>
+      <c r="L61" s="16">
+        <v>12</v>
+      </c>
+      <c r="M61" s="17"/>
+      <c r="N61" s="17"/>
+      <c r="O61" s="17"/>
       <c r="P61" s="10">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -4718,105 +4719,150 @@
       <c r="R61" s="11"/>
     </row>
     <row r="62" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="44" t="s">
+      <c r="A62" s="40" t="s">
         <v>369</v>
       </c>
-      <c r="B62" s="45" t="s">
+      <c r="B62" s="64" t="s">
         <v>182</v>
       </c>
-      <c r="C62" s="45" t="s">
-        <v>200</v>
-      </c>
-      <c r="D62" s="45" t="s">
-        <v>201</v>
-      </c>
-      <c r="E62" s="45" t="s">
-        <v>402</v>
-      </c>
-      <c r="F62" s="44" t="s">
-        <v>403</v>
-      </c>
-      <c r="G62" s="44"/>
-      <c r="H62" s="44"/>
-      <c r="I62" s="44" t="s">
-        <v>404</v>
-      </c>
-      <c r="J62" s="44" t="s">
-        <v>405</v>
-      </c>
-      <c r="K62" s="46">
-        <v>0.95</v>
-      </c>
-      <c r="L62" s="47">
-        <v>12</v>
-      </c>
-      <c r="M62" s="48"/>
-      <c r="N62" s="48"/>
-      <c r="O62" s="48"/>
-      <c r="P62" s="49">
+      <c r="C62" s="64" t="s">
+        <v>197</v>
+      </c>
+      <c r="D62" s="64" t="s">
+        <v>198</v>
+      </c>
+      <c r="E62" s="64" t="s">
+        <v>398</v>
+      </c>
+      <c r="F62" s="40" t="s">
+        <v>399</v>
+      </c>
+      <c r="G62" s="40"/>
+      <c r="H62" s="40"/>
+      <c r="I62" s="40" t="s">
+        <v>400</v>
+      </c>
+      <c r="J62" s="40" t="s">
+        <v>401</v>
+      </c>
+      <c r="K62" s="41">
+        <v>1</v>
+      </c>
+      <c r="L62" s="42">
+        <v>12</v>
+      </c>
+      <c r="M62" s="43"/>
+      <c r="N62" s="43"/>
+      <c r="O62" s="43">
+        <v>1</v>
+      </c>
+      <c r="P62" s="10">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Q62" s="11"/>
       <c r="R62" s="11"/>
     </row>
-    <row r="63" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="45" t="s">
-        <v>226</v>
+    <row r="63" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="44" t="s">
+        <v>369</v>
       </c>
       <c r="B63" s="45" t="s">
-        <v>407</v>
+        <v>182</v>
       </c>
       <c r="C63" s="45" t="s">
-        <v>406</v>
+        <v>200</v>
       </c>
       <c r="D63" s="45" t="s">
-        <v>408</v>
-      </c>
-      <c r="E63" s="45"/>
-      <c r="F63" s="45"/>
-      <c r="G63" s="45"/>
-      <c r="H63" s="45"/>
-      <c r="I63" s="45"/>
-      <c r="J63" s="45"/>
-      <c r="K63" s="52">
-        <v>1.5</v>
-      </c>
-      <c r="L63" s="53">
-        <v>12</v>
-      </c>
-      <c r="M63" s="50"/>
-      <c r="N63" s="50"/>
-      <c r="O63" s="50"/>
-      <c r="P63" s="51">
+        <v>201</v>
+      </c>
+      <c r="E63" s="45" t="s">
+        <v>402</v>
+      </c>
+      <c r="F63" s="44" t="s">
+        <v>403</v>
+      </c>
+      <c r="G63" s="44"/>
+      <c r="H63" s="44"/>
+      <c r="I63" s="44" t="s">
+        <v>404</v>
+      </c>
+      <c r="J63" s="44" t="s">
+        <v>405</v>
+      </c>
+      <c r="K63" s="46">
+        <v>0.95</v>
+      </c>
+      <c r="L63" s="47">
+        <v>12</v>
+      </c>
+      <c r="M63" s="48"/>
+      <c r="N63" s="48"/>
+      <c r="O63" s="48"/>
+      <c r="P63" s="49">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Q63" s="11"/>
-      <c r="R63" s="28"/>
+      <c r="R63" s="11"/>
     </row>
     <row r="64" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="31"/>
-      <c r="B64" s="31"/>
-      <c r="C64" s="31"/>
-      <c r="D64" s="31"/>
-      <c r="E64" s="31"/>
-      <c r="F64" s="31"/>
-      <c r="G64" s="31"/>
-      <c r="H64" s="31"/>
-      <c r="I64" s="31"/>
-      <c r="J64" s="31"/>
-      <c r="K64" s="10"/>
-      <c r="L64" s="32"/>
-      <c r="M64" s="11"/>
-      <c r="N64" s="11"/>
-      <c r="O64" s="11"/>
-      <c r="P64" s="33"/>
+      <c r="A64" s="45" t="s">
+        <v>226</v>
+      </c>
+      <c r="B64" s="45" t="s">
+        <v>407</v>
+      </c>
+      <c r="C64" s="45" t="s">
+        <v>406</v>
+      </c>
+      <c r="D64" s="45" t="s">
+        <v>408</v>
+      </c>
+      <c r="E64" s="45"/>
+      <c r="F64" s="45"/>
+      <c r="G64" s="45"/>
+      <c r="H64" s="45"/>
+      <c r="I64" s="45"/>
+      <c r="J64" s="45"/>
+      <c r="K64" s="52">
+        <v>1.5</v>
+      </c>
+      <c r="L64" s="53">
+        <v>12</v>
+      </c>
+      <c r="M64" s="50"/>
+      <c r="N64" s="50"/>
+      <c r="O64" s="50"/>
+      <c r="P64" s="51">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="Q64" s="11"/>
-      <c r="R64" s="27"/>
+      <c r="R64" s="28"/>
+    </row>
+    <row r="65" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="31"/>
+      <c r="B65" s="31"/>
+      <c r="C65" s="31"/>
+      <c r="D65" s="31"/>
+      <c r="E65" s="31"/>
+      <c r="F65" s="31"/>
+      <c r="G65" s="31"/>
+      <c r="H65" s="31"/>
+      <c r="I65" s="31"/>
+      <c r="J65" s="31"/>
+      <c r="K65" s="10"/>
+      <c r="L65" s="32"/>
+      <c r="M65" s="11"/>
+      <c r="N65" s="11"/>
+      <c r="O65" s="11"/>
+      <c r="P65" s="33"/>
+      <c r="Q65" s="11"/>
+      <c r="R65" s="27"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R64" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:R65" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="M1:O1048576">
     <cfRule type="colorScale" priority="1">
       <colorScale>
@@ -4838,7 +4884,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.5" style="3" bestFit="1" customWidth="1"/>
@@ -4992,13 +5038,13 @@
         <v>34</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>35</v>
+        <v>414</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>36</v>
+        <v>415</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>37</v>
+        <v>416</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5006,27 +5052,27 @@
         <v>34</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5034,13 +5080,13 @@
         <v>41</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5048,27 +5094,27 @@
         <v>41</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5076,13 +5122,13 @@
         <v>51</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5090,13 +5136,13 @@
         <v>51</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5104,13 +5150,13 @@
         <v>51</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5118,13 +5164,13 @@
         <v>51</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5132,27 +5178,27 @@
         <v>51</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5160,13 +5206,13 @@
         <v>70</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5174,13 +5220,13 @@
         <v>70</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5188,27 +5234,27 @@
         <v>70</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5216,13 +5262,13 @@
         <v>83</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5230,13 +5276,13 @@
         <v>83</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5244,27 +5290,27 @@
         <v>83</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5272,13 +5318,13 @@
         <v>96</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5286,27 +5332,27 @@
         <v>96</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5314,27 +5360,27 @@
         <v>106</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5342,13 +5388,13 @@
         <v>113</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5356,27 +5402,27 @@
         <v>113</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5384,41 +5430,41 @@
         <v>123</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5426,13 +5472,13 @@
         <v>134</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5440,13 +5486,13 @@
         <v>134</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5454,13 +5500,13 @@
         <v>134</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5468,13 +5514,13 @@
         <v>134</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5482,13 +5528,13 @@
         <v>134</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5496,13 +5542,13 @@
         <v>134</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5510,13 +5556,13 @@
         <v>134</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5524,13 +5570,13 @@
         <v>134</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5538,27 +5584,27 @@
         <v>134</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>165</v>
+        <v>134</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5566,27 +5612,27 @@
         <v>165</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5594,13 +5640,13 @@
         <v>172</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5608,27 +5654,27 @@
         <v>172</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5636,13 +5682,13 @@
         <v>182</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5650,13 +5696,13 @@
         <v>182</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>167</v>
+        <v>187</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5664,41 +5710,41 @@
         <v>182</v>
       </c>
       <c r="B59" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B60" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="C59" s="2" t="s">
+      <c r="C60" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="D59" s="2" t="s">
+      <c r="D60" s="2" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="60" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="54" t="s">
+    <row r="61" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A61" s="54" t="s">
         <v>182</v>
       </c>
-      <c r="B60" s="54" t="s">
+      <c r="B61" s="54" t="s">
         <v>194</v>
       </c>
-      <c r="C60" s="54" t="s">
+      <c r="C61" s="54" t="s">
         <v>195</v>
       </c>
-      <c r="D60" s="54" t="s">
+      <c r="D61" s="54" t="s">
         <v>196</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="55" t="s">
-        <v>182</v>
-      </c>
-      <c r="B61" s="55" t="s">
-        <v>197</v>
-      </c>
-      <c r="C61" s="55" t="s">
-        <v>198</v>
-      </c>
-      <c r="D61" s="55" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5706,26 +5752,40 @@
         <v>182</v>
       </c>
       <c r="B62" s="55" t="s">
+        <v>197</v>
+      </c>
+      <c r="C62" s="55" t="s">
+        <v>198</v>
+      </c>
+      <c r="D62" s="55" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="55" t="s">
+        <v>182</v>
+      </c>
+      <c r="B63" s="55" t="s">
         <v>200</v>
       </c>
-      <c r="C62" s="55" t="s">
+      <c r="C63" s="55" t="s">
         <v>201</v>
       </c>
-      <c r="D62" s="55" t="s">
+      <c r="D63" s="55" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="56" t="s">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" s="56" t="s">
         <v>407</v>
       </c>
-      <c r="B63" s="56" t="s">
+      <c r="B64" s="56" t="s">
         <v>406</v>
       </c>
-      <c r="C63" s="56" t="s">
+      <c r="C64" s="56" t="s">
         <v>408</v>
       </c>
-      <c r="D63" s="56" t="s">
+      <c r="D64" s="56" t="s">
         <v>409</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update target wali & waso
</commit_message>
<xml_diff>
--- a/ssp_modeling/scenario_mapping/ssp_libya_transformation_cw_20260408.xlsx
+++ b/ssp_modeling/scenario_mapping/ssp_libya_transformation_cw_20260408.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabianfuentes/git/ssp_libya/ssp_modeling/scenario_mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD83D44B-861A-4D40-BCD7-D270172F34E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{499A0368-1192-174B-8CCA-6F985BE9674E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-51200" yWindow="-7160" windowWidth="25600" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -1545,7 +1545,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1690,9 +1690,6 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
@@ -2072,7 +2069,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:R65"/>
@@ -2096,16 +2093,16 @@
       <c r="A1" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="B1" s="58" t="s">
+      <c r="B1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="58" t="s">
+      <c r="C1" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="58" t="s">
+      <c r="D1" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="58" t="s">
+      <c r="E1" s="57" t="s">
         <v>204</v>
       </c>
       <c r="F1" s="5" t="s">
@@ -2132,7 +2129,7 @@
       <c r="M1" s="9" t="s">
         <v>412</v>
       </c>
-      <c r="N1" s="57" t="s">
+      <c r="N1" s="56" t="s">
         <v>411</v>
       </c>
       <c r="O1" s="9" t="s">
@@ -2142,7 +2139,7 @@
       <c r="Q1" s="11"/>
       <c r="R1" s="11"/>
     </row>
-    <row r="2" spans="1:18" s="4" customFormat="1" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" s="4" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>212</v>
       </c>
@@ -2181,20 +2178,20 @@
       <c r="Q2" s="11"/>
       <c r="R2" s="11"/>
     </row>
-    <row r="3" spans="1:18" s="4" customFormat="1" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" s="4" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>212</v>
       </c>
-      <c r="B3" s="59" t="s">
+      <c r="B3" s="58" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="60" t="s">
+      <c r="C3" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="60" t="s">
+      <c r="D3" s="59" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="60" t="s">
+      <c r="E3" s="59" t="s">
         <v>215</v>
       </c>
       <c r="F3" s="18" t="s">
@@ -2220,7 +2217,7 @@
       <c r="Q3" s="11"/>
       <c r="R3" s="11"/>
     </row>
-    <row r="4" spans="1:18" s="4" customFormat="1" ht="33" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:18" s="4" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
         <v>212</v>
       </c>
@@ -2265,7 +2262,7 @@
       </c>
       <c r="R4" s="11"/>
     </row>
-    <row r="5" spans="1:18" s="4" customFormat="1" ht="95.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" s="4" customFormat="1" ht="95.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
         <v>212</v>
       </c>
@@ -2308,7 +2305,7 @@
       <c r="Q5" s="11"/>
       <c r="R5" s="11"/>
     </row>
-    <row r="6" spans="1:18" s="4" customFormat="1" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" s="4" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
         <v>212</v>
       </c>
@@ -2318,7 +2315,7 @@
       <c r="C6" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="61" t="s">
+      <c r="D6" s="60" t="s">
         <v>18</v>
       </c>
       <c r="E6" s="13" t="s">
@@ -2353,20 +2350,20 @@
       <c r="Q6" s="11"/>
       <c r="R6" s="11"/>
     </row>
-    <row r="7" spans="1:18" s="4" customFormat="1" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" s="4" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="22" t="s">
         <v>226</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="62" t="s">
+      <c r="C7" s="61" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="62" t="s">
+      <c r="D7" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="E7" s="62" t="s">
+      <c r="E7" s="61" t="s">
         <v>227</v>
       </c>
       <c r="F7" s="12" t="s">
@@ -2392,7 +2389,7 @@
       <c r="Q7" s="11"/>
       <c r="R7" s="11"/>
     </row>
-    <row r="8" spans="1:18" s="4" customFormat="1" ht="31.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:18" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
         <v>226</v>
       </c>
@@ -2439,7 +2436,7 @@
       <c r="Q8" s="11"/>
       <c r="R8" s="11"/>
     </row>
-    <row r="9" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
         <v>226</v>
       </c>
@@ -2482,7 +2479,7 @@
       <c r="Q9" s="11"/>
       <c r="R9" s="11"/>
     </row>
-    <row r="10" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
         <v>226</v>
       </c>
@@ -2529,14 +2526,14 @@
       <c r="Q10" s="11"/>
       <c r="R10" s="11"/>
     </row>
-    <row r="11" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="12" t="s">
         <v>226</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="65" t="s">
+      <c r="C11" s="64" t="s">
         <v>414</v>
       </c>
       <c r="D11" s="13" t="s">
@@ -2573,14 +2570,14 @@
       </c>
       <c r="R11" s="11"/>
     </row>
-    <row r="12" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="12" t="s">
         <v>226</v>
       </c>
       <c r="B12" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="65" t="s">
+      <c r="C12" s="64" t="s">
         <v>35</v>
       </c>
       <c r="D12" s="13" t="s">
@@ -2619,14 +2616,14 @@
       </c>
       <c r="R12" s="11"/>
     </row>
-    <row r="13" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
         <v>226</v>
       </c>
       <c r="B13" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="65" t="s">
+      <c r="C13" s="64" t="s">
         <v>38</v>
       </c>
       <c r="D13" s="13" t="s">
@@ -2667,7 +2664,7 @@
       </c>
       <c r="R13" s="11"/>
     </row>
-    <row r="14" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
         <v>226</v>
       </c>
@@ -2677,10 +2674,10 @@
       <c r="C14" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="D14" s="63" t="s">
+      <c r="D14" s="62" t="s">
         <v>43</v>
       </c>
-      <c r="E14" s="63" t="s">
+      <c r="E14" s="62" t="s">
         <v>246</v>
       </c>
       <c r="F14" s="25" t="s">
@@ -2714,7 +2711,7 @@
       <c r="Q14" s="11"/>
       <c r="R14" s="11"/>
     </row>
-    <row r="15" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="12" t="s">
         <v>226</v>
       </c>
@@ -2764,7 +2761,7 @@
       </c>
       <c r="R15" s="11"/>
     </row>
-    <row r="16" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
         <v>226</v>
       </c>
@@ -2805,54 +2802,54 @@
       <c r="Q16" s="11"/>
       <c r="R16" s="11"/>
     </row>
-    <row r="17" spans="1:18" s="71" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="65" t="s">
+    <row r="17" spans="1:18" s="70" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="64" t="s">
         <v>51</v>
       </c>
-      <c r="B17" s="65" t="s">
+      <c r="B17" s="64" t="s">
         <v>51</v>
       </c>
-      <c r="C17" s="65" t="s">
+      <c r="C17" s="64" t="s">
         <v>52</v>
       </c>
-      <c r="D17" s="65" t="s">
+      <c r="D17" s="64" t="s">
         <v>53</v>
       </c>
-      <c r="E17" s="65" t="s">
+      <c r="E17" s="64" t="s">
         <v>257</v>
       </c>
-      <c r="F17" s="65" t="s">
+      <c r="F17" s="64" t="s">
         <v>258</v>
       </c>
-      <c r="G17" s="65"/>
-      <c r="H17" s="65"/>
-      <c r="I17" s="65" t="s">
+      <c r="G17" s="64"/>
+      <c r="H17" s="64"/>
+      <c r="I17" s="64" t="s">
         <v>259</v>
       </c>
-      <c r="J17" s="65" t="s">
+      <c r="J17" s="64" t="s">
         <v>260</v>
       </c>
-      <c r="K17" s="66">
+      <c r="K17" s="65">
         <v>0.5</v>
       </c>
-      <c r="L17" s="67">
-        <v>12</v>
-      </c>
-      <c r="M17" s="68"/>
-      <c r="N17" s="68">
+      <c r="L17" s="66">
+        <v>12</v>
+      </c>
+      <c r="M17" s="67"/>
+      <c r="N17" s="67">
         <v>0.1</v>
       </c>
-      <c r="O17" s="68">
+      <c r="O17" s="67">
         <v>0.5</v>
       </c>
-      <c r="P17" s="69">
+      <c r="P17" s="68">
         <f t="shared" si="1"/>
         <v>0.05</v>
       </c>
-      <c r="Q17" s="70"/>
-      <c r="R17" s="70"/>
-    </row>
-    <row r="18" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q17" s="69"/>
+      <c r="R17" s="69"/>
+    </row>
+    <row r="18" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="12" t="s">
         <v>51</v>
       </c>
@@ -2862,10 +2859,10 @@
       <c r="C18" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="D18" s="63" t="s">
+      <c r="D18" s="62" t="s">
         <v>56</v>
       </c>
-      <c r="E18" s="62" t="s">
+      <c r="E18" s="61" t="s">
         <v>261</v>
       </c>
       <c r="F18" s="25" t="s">
@@ -2895,7 +2892,7 @@
       <c r="Q18" s="11"/>
       <c r="R18" s="11"/>
     </row>
-    <row r="19" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="12" t="s">
         <v>51</v>
       </c>
@@ -2942,7 +2939,7 @@
       <c r="Q19" s="11"/>
       <c r="R19" s="11"/>
     </row>
-    <row r="20" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="12" t="s">
         <v>51</v>
       </c>
@@ -2981,7 +2978,7 @@
       <c r="Q20" s="11"/>
       <c r="R20" s="11"/>
     </row>
-    <row r="21" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="12" t="s">
         <v>51</v>
       </c>
@@ -3024,7 +3021,7 @@
       <c r="Q21" s="11"/>
       <c r="R21" s="11"/>
     </row>
-    <row r="22" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">
         <v>51</v>
       </c>
@@ -3067,7 +3064,7 @@
       <c r="Q22" s="11"/>
       <c r="R22" s="11"/>
     </row>
-    <row r="23" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="12" t="s">
         <v>212</v>
       </c>
@@ -3077,10 +3074,10 @@
       <c r="C23" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="D23" s="63" t="s">
+      <c r="D23" s="62" t="s">
         <v>72</v>
       </c>
-      <c r="E23" s="62" t="s">
+      <c r="E23" s="61" t="s">
         <v>275</v>
       </c>
       <c r="F23" s="25" t="s">
@@ -3103,17 +3100,17 @@
       <c r="M23" s="17"/>
       <c r="N23" s="17"/>
       <c r="O23" s="17"/>
-      <c r="P23" s="73">
+      <c r="P23" s="72">
         <f>K23*N23</f>
         <v>0</v>
       </c>
-      <c r="Q23" s="74">
+      <c r="Q23" s="73">
         <f>K23*O23</f>
         <v>0</v>
       </c>
       <c r="R23" s="11"/>
     </row>
-    <row r="24" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="12" t="s">
         <v>212</v>
       </c>
@@ -3156,7 +3153,7 @@
       <c r="Q24" s="11"/>
       <c r="R24" s="11"/>
     </row>
-    <row r="25" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="12" t="s">
         <v>212</v>
       </c>
@@ -3166,10 +3163,10 @@
       <c r="C25" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="D25" s="63" t="s">
+      <c r="D25" s="62" t="s">
         <v>78</v>
       </c>
-      <c r="E25" s="62" t="s">
+      <c r="E25" s="61" t="s">
         <v>283</v>
       </c>
       <c r="F25" s="25" t="s">
@@ -3200,13 +3197,13 @@
         <f>K25*N25</f>
         <v>0.2</v>
       </c>
-      <c r="Q25" s="74">
+      <c r="Q25" s="73">
         <f>K25*O25</f>
         <v>0.99998000000000009</v>
       </c>
       <c r="R25" s="11"/>
     </row>
-    <row r="26" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="12" t="s">
         <v>212</v>
       </c>
@@ -3249,7 +3246,7 @@
       <c r="Q26" s="11"/>
       <c r="R26" s="11"/>
     </row>
-    <row r="27" spans="1:18" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:18" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="12" t="s">
         <v>212</v>
       </c>
@@ -3288,7 +3285,7 @@
       <c r="Q27" s="11"/>
       <c r="R27" s="28"/>
     </row>
-    <row r="28" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="12" t="s">
         <v>212</v>
       </c>
@@ -3331,7 +3328,7 @@
       <c r="Q28" s="11"/>
       <c r="R28" s="11"/>
     </row>
-    <row r="29" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="12" t="s">
         <v>212</v>
       </c>
@@ -3370,7 +3367,7 @@
       <c r="Q29" s="11"/>
       <c r="R29" s="11"/>
     </row>
-    <row r="30" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="12" t="s">
         <v>212</v>
       </c>
@@ -3409,7 +3406,7 @@
       <c r="Q30" s="11"/>
       <c r="R30" s="11"/>
     </row>
-    <row r="31" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="12" t="s">
         <v>212</v>
       </c>
@@ -3452,7 +3449,7 @@
       <c r="Q31" s="11"/>
       <c r="R31" s="11"/>
     </row>
-    <row r="32" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="12" t="s">
         <v>212</v>
       </c>
@@ -3491,7 +3488,7 @@
       <c r="Q32" s="11"/>
       <c r="R32" s="11"/>
     </row>
-    <row r="33" spans="1:18" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:18" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="12" t="s">
         <v>212</v>
       </c>
@@ -3534,7 +3531,7 @@
       <c r="Q33" s="17"/>
       <c r="R33" s="29"/>
     </row>
-    <row r="34" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="12" t="s">
         <v>309</v>
       </c>
@@ -3573,7 +3570,7 @@
       <c r="Q34" s="11"/>
       <c r="R34" s="11"/>
     </row>
-    <row r="35" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="12" t="s">
         <v>309</v>
       </c>
@@ -3612,14 +3609,14 @@
       <c r="Q35" s="11"/>
       <c r="R35" s="11"/>
     </row>
-    <row r="36" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="12" t="s">
         <v>226</v>
       </c>
       <c r="B36" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="C36" s="72" t="s">
+      <c r="C36" s="71" t="s">
         <v>114</v>
       </c>
       <c r="D36" s="13" t="s">
@@ -3655,14 +3652,14 @@
       <c r="Q36" s="11"/>
       <c r="R36" s="11"/>
     </row>
-    <row r="37" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="12" t="s">
         <v>226</v>
       </c>
       <c r="B37" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="C37" s="72" t="s">
+      <c r="C37" s="71" t="s">
         <v>117</v>
       </c>
       <c r="D37" s="13" t="s">
@@ -3698,7 +3695,7 @@
       <c r="Q37" s="11"/>
       <c r="R37" s="11"/>
     </row>
-    <row r="38" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="12" t="s">
         <v>226</v>
       </c>
@@ -3737,7 +3734,7 @@
       <c r="Q38" s="11"/>
       <c r="R38" s="11"/>
     </row>
-    <row r="39" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="12" t="s">
         <v>212</v>
       </c>
@@ -3776,7 +3773,7 @@
       <c r="Q39" s="11"/>
       <c r="R39" s="11"/>
     </row>
-    <row r="40" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="12" t="s">
         <v>212</v>
       </c>
@@ -4299,7 +4296,7 @@
       <c r="Q51" s="11"/>
       <c r="R51" s="11"/>
     </row>
-    <row r="52" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="12" t="s">
         <v>51</v>
       </c>
@@ -4338,7 +4335,7 @@
       <c r="Q52" s="11"/>
       <c r="R52" s="11"/>
     </row>
-    <row r="53" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="12" t="s">
         <v>51</v>
       </c>
@@ -4383,7 +4380,7 @@
       <c r="Q53" s="11"/>
       <c r="R53" s="11"/>
     </row>
-    <row r="54" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="12" t="s">
         <v>369</v>
       </c>
@@ -4417,16 +4414,17 @@
         <v>12</v>
       </c>
       <c r="M54" s="17"/>
-      <c r="N54" s="17"/>
-      <c r="O54" s="17"/>
-      <c r="P54" s="10" t="e">
-        <f t="shared" si="1"/>
-        <v>#VALUE!</v>
-      </c>
+      <c r="N54" s="17">
+        <v>1</v>
+      </c>
+      <c r="O54" s="17">
+        <v>1</v>
+      </c>
+      <c r="P54" s="10"/>
       <c r="Q54" s="11"/>
       <c r="R54" s="11"/>
     </row>
-    <row r="55" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="12" t="s">
         <v>369</v>
       </c>
@@ -4462,14 +4460,11 @@
       <c r="M55" s="17"/>
       <c r="N55" s="17"/>
       <c r="O55" s="17"/>
-      <c r="P55" s="10" t="e">
-        <f t="shared" si="1"/>
-        <v>#VALUE!</v>
-      </c>
+      <c r="P55" s="10"/>
       <c r="Q55" s="11"/>
       <c r="R55" s="11"/>
     </row>
-    <row r="56" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="12" t="s">
         <v>369</v>
       </c>
@@ -4503,20 +4498,13 @@
         <v>12</v>
       </c>
       <c r="M56" s="17"/>
-      <c r="N56" s="17">
-        <v>0.1</v>
-      </c>
-      <c r="O56" s="17">
-        <v>0.2</v>
-      </c>
-      <c r="P56" s="10" t="e">
-        <f t="shared" si="1"/>
-        <v>#VALUE!</v>
-      </c>
+      <c r="N56" s="17"/>
+      <c r="O56" s="17"/>
+      <c r="P56" s="10"/>
       <c r="Q56" s="11"/>
       <c r="R56" s="11"/>
     </row>
-    <row r="57" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="12" t="s">
         <v>369</v>
       </c>
@@ -4550,18 +4538,20 @@
         <v>12</v>
       </c>
       <c r="M57" s="17"/>
-      <c r="N57" s="17"/>
+      <c r="N57" s="17">
+        <v>0.45</v>
+      </c>
       <c r="O57" s="17">
-        <v>1</v>
+        <v>0.45</v>
       </c>
       <c r="P57" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>K57*N57</f>
+        <v>0.13500000000000001</v>
       </c>
       <c r="Q57" s="11"/>
       <c r="R57" s="11"/>
     </row>
-    <row r="58" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="12" t="s">
         <v>369</v>
       </c>
@@ -4591,18 +4581,17 @@
         <v>12</v>
       </c>
       <c r="M58" s="17"/>
-      <c r="N58" s="17"/>
+      <c r="N58" s="17">
+        <v>1</v>
+      </c>
       <c r="O58" s="17">
         <v>1</v>
       </c>
-      <c r="P58" s="10" t="e">
-        <f t="shared" si="1"/>
-        <v>#VALUE!</v>
-      </c>
+      <c r="P58" s="10"/>
       <c r="Q58" s="11"/>
       <c r="R58" s="11"/>
     </row>
-    <row r="59" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="12" t="s">
         <v>369</v>
       </c>
@@ -4612,10 +4601,10 @@
       <c r="C59" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="D59" s="62" t="s">
+      <c r="D59" s="61" t="s">
         <v>167</v>
       </c>
-      <c r="E59" s="62" t="s">
+      <c r="E59" s="61" t="s">
         <v>390</v>
       </c>
       <c r="F59" s="22" t="s">
@@ -4636,18 +4625,20 @@
         <v>12</v>
       </c>
       <c r="M59" s="17"/>
-      <c r="N59" s="17"/>
+      <c r="N59" s="17">
+        <v>0.1</v>
+      </c>
       <c r="O59" s="17">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="P59" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" ref="P59:P63" si="4">K59*N59</f>
+        <v>8.5000000000000006E-2</v>
       </c>
       <c r="Q59" s="11"/>
       <c r="R59" s="11"/>
     </row>
-    <row r="60" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="12" t="s">
         <v>369</v>
       </c>
@@ -4677,18 +4668,20 @@
         <v>12</v>
       </c>
       <c r="M60" s="17"/>
-      <c r="N60" s="17"/>
+      <c r="N60" s="17">
+        <v>0.1</v>
+      </c>
       <c r="O60" s="17">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="P60" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>8.5000000000000006E-2</v>
       </c>
       <c r="Q60" s="11"/>
       <c r="R60" s="11"/>
     </row>
-    <row r="61" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="12" t="s">
         <v>369</v>
       </c>
@@ -4721,26 +4714,26 @@
       <c r="N61" s="17"/>
       <c r="O61" s="17"/>
       <c r="P61" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="Q61" s="11"/>
       <c r="R61" s="11"/>
     </row>
-    <row r="62" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="40" t="s">
         <v>369</v>
       </c>
-      <c r="B62" s="64" t="s">
+      <c r="B62" s="63" t="s">
         <v>182</v>
       </c>
-      <c r="C62" s="64" t="s">
+      <c r="C62" s="63" t="s">
         <v>197</v>
       </c>
-      <c r="D62" s="64" t="s">
+      <c r="D62" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="E62" s="64" t="s">
+      <c r="E62" s="63" t="s">
         <v>398</v>
       </c>
       <c r="F62" s="40" t="s">
@@ -4761,18 +4754,20 @@
         <v>12</v>
       </c>
       <c r="M62" s="43"/>
-      <c r="N62" s="43"/>
+      <c r="N62" s="43">
+        <v>0.1</v>
+      </c>
       <c r="O62" s="43">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="P62" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>0.1</v>
       </c>
       <c r="Q62" s="11"/>
       <c r="R62" s="11"/>
     </row>
-    <row r="63" spans="1:18" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="44" t="s">
         <v>369</v>
       </c>
@@ -4808,14 +4803,14 @@
       <c r="M63" s="48"/>
       <c r="N63" s="48"/>
       <c r="O63" s="48"/>
-      <c r="P63" s="49">
-        <f t="shared" si="1"/>
+      <c r="P63" s="10">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="Q63" s="11"/>
       <c r="R63" s="11"/>
     </row>
-    <row r="64" spans="1:18" ht="18.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="45" t="s">
         <v>226</v>
       </c>
@@ -4834,23 +4829,23 @@
       <c r="H64" s="45"/>
       <c r="I64" s="45"/>
       <c r="J64" s="45"/>
-      <c r="K64" s="52">
+      <c r="K64" s="51">
         <v>1.5</v>
       </c>
-      <c r="L64" s="53">
-        <v>12</v>
-      </c>
-      <c r="M64" s="50"/>
-      <c r="N64" s="50"/>
-      <c r="O64" s="50"/>
-      <c r="P64" s="51">
+      <c r="L64" s="52">
+        <v>12</v>
+      </c>
+      <c r="M64" s="49"/>
+      <c r="N64" s="49"/>
+      <c r="O64" s="49"/>
+      <c r="P64" s="50">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Q64" s="11"/>
       <c r="R64" s="28"/>
     </row>
-    <row r="65" spans="1:18" ht="18.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="31"/>
       <c r="B65" s="31"/>
       <c r="C65" s="31"/>
@@ -4871,14 +4866,7 @@
       <c r="R65" s="27"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R65" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="TRDE"/>
-        <filter val="TRNS"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:R65" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="M1:O1048576">
     <cfRule type="colorScale" priority="1">
       <colorScale>
@@ -5750,58 +5738,58 @@
       </c>
     </row>
     <row r="61" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="54" t="s">
+      <c r="A61" s="53" t="s">
         <v>182</v>
       </c>
-      <c r="B61" s="54" t="s">
+      <c r="B61" s="53" t="s">
         <v>194</v>
       </c>
-      <c r="C61" s="54" t="s">
+      <c r="C61" s="53" t="s">
         <v>195</v>
       </c>
-      <c r="D61" s="54" t="s">
+      <c r="D61" s="53" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="55" t="s">
+      <c r="A62" s="54" t="s">
         <v>182</v>
       </c>
-      <c r="B62" s="55" t="s">
+      <c r="B62" s="54" t="s">
         <v>197</v>
       </c>
-      <c r="C62" s="55" t="s">
+      <c r="C62" s="54" t="s">
         <v>198</v>
       </c>
-      <c r="D62" s="55" t="s">
+      <c r="D62" s="54" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="55" t="s">
+      <c r="A63" s="54" t="s">
         <v>182</v>
       </c>
-      <c r="B63" s="55" t="s">
+      <c r="B63" s="54" t="s">
         <v>200</v>
       </c>
-      <c r="C63" s="55" t="s">
+      <c r="C63" s="54" t="s">
         <v>201</v>
       </c>
-      <c r="D63" s="55" t="s">
+      <c r="D63" s="54" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" s="56" t="s">
+      <c r="A64" s="55" t="s">
         <v>407</v>
       </c>
-      <c r="B64" s="56" t="s">
+      <c r="B64" s="55" t="s">
         <v>406</v>
       </c>
-      <c r="C64" s="56" t="s">
+      <c r="C64" s="55" t="s">
         <v>408</v>
       </c>
-      <c r="D64" s="56" t="s">
+      <c r="D64" s="55" t="s">
         <v>409</v>
       </c>
     </row>
@@ -5888,10 +5876,10 @@
       </c>
     </row>
     <row r="16" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I16" s="75">
+      <c r="I16" s="74">
         <v>8</v>
       </c>
-      <c r="J16" s="75">
+      <c r="J16" s="74">
         <f t="shared" si="0"/>
         <v>2023</v>
       </c>
@@ -5996,10 +5984,10 @@
       </c>
     </row>
     <row r="28" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I28" s="75">
+      <c r="I28" s="74">
         <v>20</v>
       </c>
-      <c r="J28" s="75">
+      <c r="J28" s="74">
         <f t="shared" si="0"/>
         <v>2035</v>
       </c>

</xml_diff>

<commit_message>
adj venting, fgt, flare prop
</commit_message>
<xml_diff>
--- a/ssp_modeling/scenario_mapping/ssp_libya_transformation_cw_20260408.xlsx
+++ b/ssp_modeling/scenario_mapping/ssp_libya_transformation_cw_20260408.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabianfuentes/git/ssp_libya/ssp_modeling/scenario_mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52917AC6-9EC5-1B4B-A9E1-6043B80238A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DEFDE13-0DE4-C947-AC3F-52809E389B11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-43680" yWindow="-7160" windowWidth="32000" windowHeight="27620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -2093,7 +2093,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:S65"/>
@@ -2164,7 +2164,7 @@
       <c r="R1" s="11"/>
       <c r="S1" s="11"/>
     </row>
-    <row r="2" spans="1:19" s="4" customFormat="1" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:19" s="4" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>212</v>
       </c>
@@ -2204,7 +2204,7 @@
       <c r="R2" s="11"/>
       <c r="S2" s="11"/>
     </row>
-    <row r="3" spans="1:19" s="4" customFormat="1" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:19" s="4" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>212</v>
       </c>
@@ -2244,7 +2244,7 @@
       <c r="R3" s="11"/>
       <c r="S3" s="11"/>
     </row>
-    <row r="4" spans="1:19" s="4" customFormat="1" ht="86" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:19" s="4" customFormat="1" ht="86" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
         <v>212</v>
       </c>
@@ -2290,7 +2290,7 @@
       </c>
       <c r="S4" s="11"/>
     </row>
-    <row r="5" spans="1:19" s="4" customFormat="1" ht="95.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:19" s="4" customFormat="1" ht="95.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
         <v>212</v>
       </c>
@@ -2330,7 +2330,7 @@
       <c r="R5" s="11"/>
       <c r="S5" s="11"/>
     </row>
-    <row r="6" spans="1:19" s="4" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:19" s="4" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
         <v>212</v>
       </c>
@@ -2376,7 +2376,7 @@
       <c r="R6" s="11"/>
       <c r="S6" s="11"/>
     </row>
-    <row r="7" spans="1:19" s="4" customFormat="1" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:19" s="4" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="22" t="s">
         <v>226</v>
       </c>
@@ -2416,7 +2416,7 @@
       <c r="R7" s="11"/>
       <c r="S7" s="11"/>
     </row>
-    <row r="8" spans="1:19" s="4" customFormat="1" ht="31.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:19" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
         <v>226</v>
       </c>
@@ -2464,7 +2464,7 @@
       <c r="R8" s="11"/>
       <c r="S8" s="11"/>
     </row>
-    <row r="9" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
         <v>226</v>
       </c>
@@ -2508,7 +2508,7 @@
       <c r="R9" s="11"/>
       <c r="S9" s="11"/>
     </row>
-    <row r="10" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
         <v>226</v>
       </c>
@@ -2556,7 +2556,7 @@
       <c r="R10" s="11"/>
       <c r="S10" s="11"/>
     </row>
-    <row r="11" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="12" t="s">
         <v>226</v>
       </c>
@@ -2581,27 +2581,27 @@
         <v>0.5</v>
       </c>
       <c r="L11" s="16">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="M11" s="17"/>
       <c r="N11" s="17">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="O11" s="17">
-        <v>1</v>
+        <v>1.9</v>
       </c>
       <c r="P11" s="10"/>
       <c r="Q11" s="10">
         <f>K11*N11</f>
-        <v>0.375</v>
+        <v>0.5</v>
       </c>
       <c r="R11" s="10">
         <f>K11*O11</f>
-        <v>0.5</v>
+        <v>0.95</v>
       </c>
       <c r="S11" s="11"/>
     </row>
-    <row r="12" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="12" t="s">
         <v>226</v>
       </c>
@@ -2635,7 +2635,7 @@
         <v>0.8</v>
       </c>
       <c r="O12" s="17">
-        <v>1.24</v>
+        <v>1.25</v>
       </c>
       <c r="P12" s="10"/>
       <c r="Q12" s="10">
@@ -2644,11 +2644,11 @@
       </c>
       <c r="R12" s="10">
         <f>K12*O12</f>
-        <v>0.99199999999999999</v>
+        <v>1</v>
       </c>
       <c r="S12" s="11"/>
     </row>
-    <row r="13" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
         <v>226</v>
       </c>
@@ -2700,7 +2700,7 @@
       </c>
       <c r="S13" s="11"/>
     </row>
-    <row r="14" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
         <v>226</v>
       </c>
@@ -2748,7 +2748,7 @@
       <c r="R14" s="11"/>
       <c r="S14" s="11"/>
     </row>
-    <row r="15" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="12" t="s">
         <v>226</v>
       </c>
@@ -2799,7 +2799,7 @@
       </c>
       <c r="S15" s="11"/>
     </row>
-    <row r="16" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
         <v>226</v>
       </c>
@@ -2841,7 +2841,7 @@
       <c r="R16" s="11"/>
       <c r="S16" s="11"/>
     </row>
-    <row r="17" spans="1:19" s="69" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:19" s="69" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="63" t="s">
         <v>51</v>
       </c>
@@ -2889,7 +2889,7 @@
       <c r="R17" s="68"/>
       <c r="S17" s="68"/>
     </row>
-    <row r="18" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="12" t="s">
         <v>51</v>
       </c>
@@ -2933,7 +2933,7 @@
       <c r="R18" s="11"/>
       <c r="S18" s="11"/>
     </row>
-    <row r="19" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="12" t="s">
         <v>51</v>
       </c>
@@ -2981,7 +2981,7 @@
       <c r="R19" s="11"/>
       <c r="S19" s="11"/>
     </row>
-    <row r="20" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="12" t="s">
         <v>51</v>
       </c>
@@ -3021,7 +3021,7 @@
       <c r="R20" s="11"/>
       <c r="S20" s="11"/>
     </row>
-    <row r="21" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="12" t="s">
         <v>51</v>
       </c>
@@ -3065,7 +3065,7 @@
       <c r="R21" s="11"/>
       <c r="S21" s="11"/>
     </row>
-    <row r="22" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">
         <v>51</v>
       </c>
@@ -3109,7 +3109,7 @@
       <c r="R22" s="11"/>
       <c r="S22" s="11"/>
     </row>
-    <row r="23" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="12" t="s">
         <v>212</v>
       </c>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="S23" s="11"/>
     </row>
-    <row r="24" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="12" t="s">
         <v>212</v>
       </c>
@@ -3200,7 +3200,7 @@
       <c r="R24" s="11"/>
       <c r="S24" s="11"/>
     </row>
-    <row r="25" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="12" t="s">
         <v>212</v>
       </c>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="S25" s="11"/>
     </row>
-    <row r="26" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="12" t="s">
         <v>212</v>
       </c>
@@ -3295,7 +3295,7 @@
       <c r="R26" s="11"/>
       <c r="S26" s="11"/>
     </row>
-    <row r="27" spans="1:19" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:19" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="12" t="s">
         <v>212</v>
       </c>
@@ -3339,7 +3339,7 @@
       <c r="R27" s="11"/>
       <c r="S27" s="28"/>
     </row>
-    <row r="28" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="12" t="s">
         <v>212</v>
       </c>
@@ -3383,7 +3383,7 @@
       <c r="R28" s="11"/>
       <c r="S28" s="11"/>
     </row>
-    <row r="29" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="12" t="s">
         <v>212</v>
       </c>
@@ -3427,7 +3427,7 @@
       <c r="R29" s="11"/>
       <c r="S29" s="11"/>
     </row>
-    <row r="30" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="12" t="s">
         <v>212</v>
       </c>
@@ -3467,7 +3467,7 @@
       <c r="R30" s="11"/>
       <c r="S30" s="11"/>
     </row>
-    <row r="31" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="12" t="s">
         <v>212</v>
       </c>
@@ -3511,7 +3511,7 @@
       <c r="R31" s="11"/>
       <c r="S31" s="11"/>
     </row>
-    <row r="32" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="12" t="s">
         <v>212</v>
       </c>
@@ -3551,7 +3551,7 @@
       <c r="R32" s="11"/>
       <c r="S32" s="11"/>
     </row>
-    <row r="33" spans="1:19" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:19" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="12" t="s">
         <v>212</v>
       </c>
@@ -3597,7 +3597,7 @@
       <c r="R33" s="17"/>
       <c r="S33" s="29"/>
     </row>
-    <row r="34" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="12" t="s">
         <v>309</v>
       </c>
@@ -3637,7 +3637,7 @@
       <c r="R34" s="11"/>
       <c r="S34" s="11"/>
     </row>
-    <row r="35" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="12" t="s">
         <v>309</v>
       </c>
@@ -3677,7 +3677,7 @@
       <c r="R35" s="11"/>
       <c r="S35" s="11"/>
     </row>
-    <row r="36" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="12" t="s">
         <v>226</v>
       </c>
@@ -3721,7 +3721,7 @@
       <c r="R36" s="11"/>
       <c r="S36" s="11"/>
     </row>
-    <row r="37" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="12" t="s">
         <v>226</v>
       </c>
@@ -3765,7 +3765,7 @@
       <c r="R37" s="11"/>
       <c r="S37" s="11"/>
     </row>
-    <row r="38" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="12" t="s">
         <v>226</v>
       </c>
@@ -3805,7 +3805,7 @@
       <c r="R38" s="11"/>
       <c r="S38" s="11"/>
     </row>
-    <row r="39" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="12" t="s">
         <v>212</v>
       </c>
@@ -3849,7 +3849,7 @@
       <c r="R39" s="11"/>
       <c r="S39" s="11"/>
     </row>
-    <row r="40" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="12" t="s">
         <v>212</v>
       </c>
@@ -3893,7 +3893,7 @@
       <c r="R40" s="11"/>
       <c r="S40" s="11"/>
     </row>
-    <row r="41" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="12" t="s">
         <v>226</v>
       </c>
@@ -3940,7 +3940,7 @@
       </c>
       <c r="S41" s="11"/>
     </row>
-    <row r="42" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="12" t="s">
         <v>226</v>
       </c>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="S42" s="11"/>
     </row>
-    <row r="43" spans="1:19" s="4" customFormat="1" ht="18.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:19" s="4" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="12" t="s">
         <v>226</v>
       </c>
@@ -4039,7 +4039,7 @@
       <c r="R43" s="11"/>
       <c r="S43" s="11"/>
     </row>
-    <row r="44" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="12" t="s">
         <v>226</v>
       </c>
@@ -4079,7 +4079,7 @@
       <c r="R44" s="11"/>
       <c r="S44" s="11"/>
     </row>
-    <row r="45" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="12" t="s">
         <v>226</v>
       </c>
@@ -4123,7 +4123,7 @@
       <c r="R45" s="11"/>
       <c r="S45" s="11"/>
     </row>
-    <row r="46" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="12" t="s">
         <v>226</v>
       </c>
@@ -4167,7 +4167,7 @@
       <c r="R46" s="11"/>
       <c r="S46" s="11"/>
     </row>
-    <row r="47" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="12" t="s">
         <v>226</v>
       </c>
@@ -4215,7 +4215,7 @@
       <c r="R47" s="11"/>
       <c r="S47" s="11"/>
     </row>
-    <row r="48" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="12" t="s">
         <v>226</v>
       </c>
@@ -4255,7 +4255,7 @@
       <c r="R48" s="11"/>
       <c r="S48" s="11"/>
     </row>
-    <row r="49" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="12" t="s">
         <v>226</v>
       </c>
@@ -4299,7 +4299,7 @@
       <c r="R49" s="11"/>
       <c r="S49" s="11"/>
     </row>
-    <row r="50" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="12" t="s">
         <v>226</v>
       </c>
@@ -4347,7 +4347,7 @@
       <c r="R50" s="11"/>
       <c r="S50" s="11"/>
     </row>
-    <row r="51" spans="1:19" s="4" customFormat="1" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:19" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="12" t="s">
         <v>226</v>
       </c>
@@ -4916,7 +4916,7 @@
       <c r="R63" s="11"/>
       <c r="S63" s="11"/>
     </row>
-    <row r="64" spans="1:19" ht="18.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:19" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="45" t="s">
         <v>226</v>
       </c>
@@ -4952,7 +4952,7 @@
       <c r="R64" s="11"/>
       <c r="S64" s="28"/>
     </row>
-    <row r="65" spans="1:19" ht="18.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:19" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="31"/>
       <c r="B65" s="31"/>
       <c r="C65" s="31"/>
@@ -4974,15 +4974,7 @@
       <c r="S65" s="27"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S65" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="TRWW"/>
-        <filter val="WALI"/>
-        <filter val="WASO"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:S65" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="M1:O1048576">
     <cfRule type="colorScale" priority="1">
       <colorScale>

</xml_diff>